<commit_message>
Rescope BIM summary to BIM-only entries (exclude ELIA/TBU rows)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011perRKT2EmENmrFmt59Nd9
</commit_message>
<xml_diff>
--- a/BIM分錄_檢核修正版.xlsx
+++ b/BIM分錄_檢核修正版.xlsx
@@ -918,7 +918,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="220">
+  <cellXfs count="217">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1510,9 +1510,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="38" fontId="16" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="38" fontId="16" fillId="19" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1520,12 +1517,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1538,7 +1529,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="38" fontId="16" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -1625,7 +1618,7 @@
   <commentList>
     <comment ref="F21" authorId="0" shapeId="0">
       <text>
-        <t>修正：原寫死5；毛利=收入105.26-成本100=5.26，寫死造成分錄借貸差0.263</t>
+        <t>修正：原寫死5；毛利=收入105.26-成本100=5.26，寫死使本筆借貸差0.263</t>
       </text>
     </comment>
     <comment ref="K21" authorId="0" shapeId="0">
@@ -1633,84 +1626,369 @@
         <t>修正：同F21</t>
       </text>
     </comment>
+    <comment ref="E50" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C50,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J50" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H50,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O50" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M50,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T50" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R50,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="E51" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C51,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J51" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H51,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O51" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M51,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T51" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R51,$U$2:$U$47)</t>
+      </text>
+    </comment>
     <comment ref="E52" authorId="0" shapeId="0">
       <text>
-        <t>修正：範圍原為 =SUMIF($D$2:$D$34,$C52,$F$2:$F$34)，漏掉第38-39列ELIA沖銷，統一到第47列</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$34,$C52,$F$2:$F$34)</t>
       </text>
     </comment>
     <comment ref="J52" authorId="0" shapeId="0">
       <text>
-        <t>修正：範圍原為 =SUMIF($I$2:$I$34,$H52,$K$2:$K$34)，漏掉第38-39列ELIA沖銷，統一到第47列</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$34,$H52,$K$2:$K$34)</t>
       </text>
     </comment>
     <comment ref="O52" authorId="0" shapeId="0">
       <text>
-        <t>修正：範圍原為 =SUMIF($N$2:$N$34,$M52,$P$2:$P$34)，漏掉第38-39列ELIA沖銷，統一到第47列</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$34,$M52,$P$2:$P$34)</t>
       </text>
     </comment>
     <comment ref="T52" authorId="0" shapeId="0">
       <text>
-        <t>修正：範圍原為 =SUMIF($S$2:$S$34,$R52,$U$2:$U$34)，漏掉第38-39列ELIA沖銷，統一到第47列</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$34,$R52,$U$2:$U$34)</t>
+      </text>
+    </comment>
+    <comment ref="E53" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C53,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J53" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H53,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O53" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M53,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T53" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R53,$U$2:$U$47)</t>
       </text>
     </comment>
     <comment ref="E54" authorId="0" shapeId="0">
       <text>
-        <t>修正：原只抓11430000(BIM端往來120)，漏TBU端12872012(-120)，B/S多列120</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C54,$F$2:$F$47)</t>
       </text>
     </comment>
     <comment ref="J54" authorId="0" shapeId="0">
       <text>
-        <t>修正：與其他三欄同式；外案無12872012分錄，數值不變</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H54,$K$2:$K$47)</t>
       </text>
     </comment>
     <comment ref="O54" authorId="0" shapeId="0">
       <text>
-        <t>修正：原只抓11430000(BIM端往來120)，漏TBU端12872012(-120)，B/S多列120</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M54,$P$2:$P$47)</t>
       </text>
     </comment>
     <comment ref="T54" authorId="0" shapeId="0">
       <text>
-        <t>修正：原只抓11430000(BIM端往來120)，漏TBU端12872012(-120)，B/S多列120</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R54,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="E55" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C55,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J55" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H55,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O55" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M55,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T55" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R55,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="E56" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C56,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J56" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H56,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O56" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M56,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T56" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R56,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="E57" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C57,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J57" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H57,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O57" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M57,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T57" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R57,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="E58" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C58,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J58" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H58,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O58" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M58,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T58" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R58,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="E59" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C59,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J59" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H59,$K$2:$K$47)</t>
       </text>
     </comment>
     <comment ref="O59" authorId="0" shapeId="0">
       <text>
-        <t>修正：補漏列科目 55110095 承攬工程成本-其他</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$34,$M59,$P$2:$P$34)</t>
       </text>
     </comment>
     <comment ref="T59" authorId="0" shapeId="0">
       <text>
-        <t>修正：補漏列科目 62370030 勞務費-其他</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$34,$R59,$U$2:$U$34)</t>
       </text>
     </comment>
     <comment ref="E60" authorId="0" shapeId="0">
       <text>
-        <t>修正：補漏列科目 55110095 承攬工程成本-其他</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C60,$F$2:$F$47)</t>
       </text>
     </comment>
-    <comment ref="E61" authorId="0" shapeId="0">
+    <comment ref="J60" authorId="0" shapeId="0">
       <text>
-        <t>修正：補漏列科目 63670100 工程工務所費用-其他費用</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H60,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O60" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M60,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T60" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R60,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="J61" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H61,$K$2:$K$47)</t>
       </text>
     </comment>
     <comment ref="O61" authorId="0" shapeId="0">
       <text>
-        <t>修正：補漏列科目 63670100 工程工務所費用-其他費用</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M61,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T61" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R61,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="E62" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C62,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J62" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H62,$K$2:$K$47)</t>
       </text>
     </comment>
     <comment ref="O62" authorId="0" shapeId="0">
       <text>
-        <t>修正：範圍原為 =SUMIF($N$2:$N$36,$M62,$P$2:$P$36)，漏掉第38-39列ELIA沖銷，統一到第47列</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$36,$M62,$P$2:$P$36)</t>
       </text>
     </comment>
     <comment ref="T62" authorId="0" shapeId="0">
       <text>
-        <t>修正：範圍原為 =SUMIF($S$2:$S$36,$R62,$U$2:$U$36)，漏掉第38-39列ELIA沖銷，統一到第47列</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$36,$R62,$U$2:$U$36)</t>
+      </text>
+    </comment>
+    <comment ref="E63" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C63,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J63" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H63,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O63" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M63,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T63" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R63,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="J64" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H64,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O64" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M64,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T64" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R64,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="J65" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H65,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O65" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M65,$P$2:$P$47)</t>
       </text>
     </comment>
     <comment ref="T65" authorId="0" shapeId="0">
       <text>
-        <t>修正：範圍原為 =SUMIF($S$2:$S$37,$R65,$U$2:$U$37)，漏掉第38-39列ELIA沖銷，統一到第47列</t>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$37,$R65,$U$2:$U$37)</t>
+      </text>
+    </comment>
+    <comment ref="E66" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C66,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J66" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H66,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O66" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M66,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T66" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R66,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="E67" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C67,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J67" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H67,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O67" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M67,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T67" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R67,$U$2:$U$47)</t>
+      </text>
+    </comment>
+    <comment ref="E68" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C68,$F$2:$F$47)</t>
+      </text>
+    </comment>
+    <comment ref="J68" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H68,$K$2:$K$47)</t>
+      </text>
+    </comment>
+    <comment ref="O68" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M68,$P$2:$P$47)</t>
+      </text>
+    </comment>
+    <comment ref="T68" authorId="0" shapeId="0">
+      <text>
+        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R68,$U$2:$U$47)</t>
       </text>
     </comment>
   </commentList>
@@ -4466,7 +4744,7 @@
         </is>
       </c>
       <c r="E50" s="110">
-        <f>SUMIF($D$2:$D$47,$C50,$F$2:$F$47)</f>
+        <f>SUMIF($D$4:$D$10,$C50,$F$4:$F$10)+SUMIF($D$16:$D$22,$C50,$F$16:$F$22)+SUMIF($D$31:$D$33,$C50,$F$31:$F$33)+SUMIF($D$42:$D$46,$C50,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F50" s="197">
@@ -4486,7 +4764,7 @@
         </is>
       </c>
       <c r="J50" s="110">
-        <f>SUMIF($I$2:$I$47,$H50,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H50,$K$4:$K$10)+SUMIF($I$16:$I$22,$H50,$K$16:$K$22)+SUMIF($I$31:$I$33,$H50,$K$31:$K$33)+SUMIF($I$42:$I$46,$H50,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K50" s="197">
@@ -4506,7 +4784,7 @@
         </is>
       </c>
       <c r="O50" s="110">
-        <f>SUMIF($N$2:$N$47,$M50,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M50,$P$4:$P$10)+SUMIF($N$16:$N$22,$M50,$P$16:$P$22)+SUMIF($N$31:$N$33,$M50,$P$31:$P$33)+SUMIF($N$42:$N$46,$M50,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P50" s="197">
@@ -4526,7 +4804,7 @@
         </is>
       </c>
       <c r="T50" s="110">
-        <f>SUMIF($S$2:$S$47,$R50,$U$2:$U$47)</f>
+        <f>SUMIF($S$4:$S$10,$R50,$U$4:$U$10)+SUMIF($S$16:$S$22,$R50,$U$16:$U$22)+SUMIF($S$31:$S$33,$R50,$U$31:$U$33)+SUMIF($S$42:$S$46,$R50,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U50" s="197">
@@ -4553,8 +4831,8 @@
           <t>在建損益-承攬案</t>
         </is>
       </c>
-      <c r="E51" s="111">
-        <f>SUMIF($D$2:$D$47,$C51,$F$2:$F$47)</f>
+      <c r="E51" s="216">
+        <f>SUMIF($D$4:$D$10,$C51,$F$4:$F$10)+SUMIF($D$16:$D$22,$C51,$F$16:$F$22)+SUMIF($D$31:$D$33,$C51,$F$31:$F$33)+SUMIF($D$42:$D$46,$C51,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F51" s="201" t="n"/>
@@ -4568,7 +4846,7 @@
         </is>
       </c>
       <c r="J51" s="111">
-        <f>SUMIF($I$2:$I$47,$H51,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H51,$K$4:$K$10)+SUMIF($I$16:$I$22,$H51,$K$16:$K$22)+SUMIF($I$31:$I$33,$H51,$K$31:$K$33)+SUMIF($I$42:$I$46,$H51,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K51" s="201" t="n"/>
@@ -4582,7 +4860,7 @@
         </is>
       </c>
       <c r="O51" s="111">
-        <f>SUMIF($N$2:$N$47,$M51,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M51,$P$4:$P$10)+SUMIF($N$16:$N$22,$M51,$P$16:$P$22)+SUMIF($N$31:$N$33,$M51,$P$31:$P$33)+SUMIF($N$42:$N$46,$M51,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P51" s="201" t="n"/>
@@ -4596,7 +4874,7 @@
         </is>
       </c>
       <c r="T51" s="111">
-        <f>SUMIF($S$2:$S$47,$R51,$U$2:$U$47)</f>
+        <f>SUMIF($S$4:$S$10,$R51,$U$4:$U$10)+SUMIF($S$16:$S$22,$R51,$U$16:$U$22)+SUMIF($S$31:$S$33,$R51,$U$31:$U$33)+SUMIF($S$42:$S$46,$R51,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U51" s="201" t="n"/>
@@ -4617,12 +4895,12 @@
           <t>預收工程款</t>
         </is>
       </c>
-      <c r="E52" s="203">
-        <f>SUMIF($D$2:$D$47,$C52,$F$2:$F$47)</f>
-        <v/>
-      </c>
-      <c r="F52" s="204" t="n"/>
-      <c r="G52" s="205" t="n"/>
+      <c r="E52" s="111">
+        <f>SUMIF($D$4:$D$10,$C52,$F$4:$F$10)+SUMIF($D$16:$D$22,$C52,$F$16:$F$22)+SUMIF($D$31:$D$33,$C52,$F$31:$F$33)+SUMIF($D$42:$D$46,$C52,$F$42:$F$46)</f>
+        <v/>
+      </c>
+      <c r="F52" s="203" t="n"/>
+      <c r="G52" s="204" t="n"/>
       <c r="H52" s="13" t="n">
         <v>22640000</v>
       </c>
@@ -4631,12 +4909,12 @@
           <t>預收工程款</t>
         </is>
       </c>
-      <c r="J52" s="203">
-        <f>SUMIF($I$2:$I$47,$H52,$K$2:$K$47)</f>
-        <v/>
-      </c>
-      <c r="K52" s="204" t="n"/>
-      <c r="L52" s="205" t="n"/>
+      <c r="J52" s="111">
+        <f>SUMIF($I$4:$I$10,$H52,$K$4:$K$10)+SUMIF($I$16:$I$22,$H52,$K$16:$K$22)+SUMIF($I$31:$I$33,$H52,$K$31:$K$33)+SUMIF($I$42:$I$46,$H52,$K$42:$K$46)</f>
+        <v/>
+      </c>
+      <c r="K52" s="203" t="n"/>
+      <c r="L52" s="204" t="n"/>
       <c r="M52" s="134" t="n">
         <v>22640000</v>
       </c>
@@ -4645,12 +4923,12 @@
           <t>預收工程款</t>
         </is>
       </c>
-      <c r="O52" s="203">
-        <f>SUMIF($N$2:$N$47,$M52,$P$2:$P$47)</f>
-        <v/>
-      </c>
-      <c r="P52" s="204" t="n"/>
-      <c r="Q52" s="205" t="n"/>
+      <c r="O52" s="111">
+        <f>SUMIF($N$4:$N$10,$M52,$P$4:$P$10)+SUMIF($N$16:$N$22,$M52,$P$16:$P$22)+SUMIF($N$31:$N$33,$M52,$P$31:$P$33)+SUMIF($N$42:$N$46,$M52,$P$42:$P$46)</f>
+        <v/>
+      </c>
+      <c r="P52" s="203" t="n"/>
+      <c r="Q52" s="204" t="n"/>
       <c r="R52" s="134" t="n">
         <v>22640000</v>
       </c>
@@ -4659,12 +4937,12 @@
           <t>預收工程款</t>
         </is>
       </c>
-      <c r="T52" s="203">
-        <f>SUMIF($S$2:$S$47,$R52,$U$2:$U$47)</f>
-        <v/>
-      </c>
-      <c r="U52" s="204" t="n"/>
-      <c r="V52" s="205" t="n"/>
+      <c r="T52" s="111">
+        <f>SUMIF($S$4:$S$10,$R52,$U$4:$U$10)+SUMIF($S$16:$S$22,$R52,$U$16:$U$22)+SUMIF($S$31:$S$33,$R52,$U$31:$U$33)+SUMIF($S$42:$S$46,$R52,$U$42:$U$46)</f>
+        <v/>
+      </c>
+      <c r="U52" s="203" t="n"/>
+      <c r="V52" s="204" t="n"/>
       <c r="W52" s="79" t="n"/>
       <c r="X52" s="79" t="n"/>
       <c r="Y52" s="79" t="n"/>
@@ -4684,7 +4962,7 @@
         </is>
       </c>
       <c r="E53" s="121">
-        <f>SUMIF($D$2:$D$47,$C53,$F$2:$F$47)</f>
+        <f>SUMIF($D$4:$D$10,$C53,$F$4:$F$10)+SUMIF($D$16:$D$22,$C53,$F$16:$F$22)+SUMIF($D$31:$D$33,$C53,$F$31:$F$33)+SUMIF($D$42:$D$46,$C53,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F53" s="115">
@@ -4707,7 +4985,7 @@
         </is>
       </c>
       <c r="J53" s="121">
-        <f>SUMIF($I$2:$I$47,$H53,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H53,$K$4:$K$10)+SUMIF($I$16:$I$22,$H53,$K$16:$K$22)+SUMIF($I$31:$I$33,$H53,$K$31:$K$33)+SUMIF($I$42:$I$46,$H53,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K53" s="115">
@@ -4730,7 +5008,7 @@
         </is>
       </c>
       <c r="O53" s="121">
-        <f>SUMIF($N$2:$N$47,$M53,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M53,$P$4:$P$10)+SUMIF($N$16:$N$22,$M53,$P$16:$P$22)+SUMIF($N$31:$N$33,$M53,$P$31:$P$33)+SUMIF($N$42:$N$46,$M53,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P53" s="115">
@@ -4753,7 +5031,7 @@
         </is>
       </c>
       <c r="T53" s="121">
-        <f>SUMIF($S$2:$S$47,$R53,$U$2:$U$47)</f>
+        <f>SUMIF($S$4:$S$10,$R53,$U$4:$U$10)+SUMIF($S$16:$S$22,$R53,$U$16:$U$22)+SUMIF($S$31:$S$33,$R53,$U$31:$U$33)+SUMIF($S$42:$S$46,$R53,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U53" s="115">
@@ -4778,11 +5056,11 @@
       </c>
       <c r="D54" s="98" t="inlineStr">
         <is>
-          <t>應收帳款/內部往來(11430000+12872012淨額)</t>
-        </is>
-      </c>
-      <c r="E54" s="203">
-        <f>SUMIF($D$2:$D$47,C54,$F$2:$F$47)+SUMIF($D$2:$D$47,"12872012",$F$2:$F$47)</f>
+          <t>應收帳款</t>
+        </is>
+      </c>
+      <c r="E54" s="122">
+        <f>SUMIF($D$4:$D$10,$C54,$F$4:$F$10)+SUMIF($D$16:$D$22,$C54,$F$16:$F$22)+SUMIF($D$31:$D$33,$C54,$F$31:$F$33)+SUMIF($D$42:$D$46,$C54,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F54" s="116">
@@ -4799,11 +5077,11 @@
       </c>
       <c r="I54" s="98" t="inlineStr">
         <is>
-          <t>應收帳款/內部往來(11430000+12872012淨額)</t>
-        </is>
-      </c>
-      <c r="J54" s="203">
-        <f>SUMIF($I$2:$I$47,H54,$K$2:$K$47)+SUMIF($I$2:$I$47,"12872012",$K$2:$K$47)</f>
+          <t>應收帳款</t>
+        </is>
+      </c>
+      <c r="J54" s="122">
+        <f>SUMIF($I$4:$I$10,$H54,$K$4:$K$10)+SUMIF($I$16:$I$22,$H54,$K$16:$K$22)+SUMIF($I$31:$I$33,$H54,$K$31:$K$33)+SUMIF($I$42:$I$46,$H54,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K54" s="116">
@@ -4820,11 +5098,11 @@
       </c>
       <c r="N54" s="98" t="inlineStr">
         <is>
-          <t>應收帳款/內部往來(11430000+12872012淨額)</t>
-        </is>
-      </c>
-      <c r="O54" s="203">
-        <f>SUMIF($N$2:$N$47,M54,$P$2:$P$47)+SUMIF($N$2:$N$47,"12872012",$P$2:$P$47)</f>
+          <t>應收帳款</t>
+        </is>
+      </c>
+      <c r="O54" s="122">
+        <f>SUMIF($N$4:$N$10,$M54,$P$4:$P$10)+SUMIF($N$16:$N$22,$M54,$P$16:$P$22)+SUMIF($N$31:$N$33,$M54,$P$31:$P$33)+SUMIF($N$42:$N$46,$M54,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P54" s="116">
@@ -4841,11 +5119,11 @@
       </c>
       <c r="S54" s="98" t="inlineStr">
         <is>
-          <t>應收帳款/內部往來(11430000+12872012淨額)</t>
-        </is>
-      </c>
-      <c r="T54" s="203">
-        <f>SUMIF($S$2:$S$47,R54,$U$2:$U$47)+SUMIF($S$2:$S$47,"12872012",$U$2:$U$47)</f>
+          <t>應收帳款</t>
+        </is>
+      </c>
+      <c r="T54" s="122">
+        <f>SUMIF($S$4:$S$10,$R54,$U$4:$U$10)+SUMIF($S$16:$S$22,$R54,$U$16:$U$22)+SUMIF($S$31:$S$33,$R54,$U$31:$U$33)+SUMIF($S$42:$S$46,$R54,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U54" s="116">
@@ -4874,7 +5152,7 @@
         </is>
       </c>
       <c r="E55" s="122">
-        <f>SUMIF($D$2:$D$47,$C55,$F$2:$F$47)</f>
+        <f>SUMIF($D$4:$D$10,$C55,$F$4:$F$10)+SUMIF($D$16:$D$22,$C55,$F$16:$F$22)+SUMIF($D$31:$D$33,$C55,$F$31:$F$33)+SUMIF($D$42:$D$46,$C55,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F55" s="116">
@@ -4895,7 +5173,7 @@
         </is>
       </c>
       <c r="J55" s="122">
-        <f>SUMIF($I$2:$I$47,$H55,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H55,$K$4:$K$10)+SUMIF($I$16:$I$22,$H55,$K$16:$K$22)+SUMIF($I$31:$I$33,$H55,$K$31:$K$33)+SUMIF($I$42:$I$46,$H55,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K55" s="116">
@@ -4916,7 +5194,7 @@
         </is>
       </c>
       <c r="O55" s="122">
-        <f>SUMIF($N$2:$N$47,$M55,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M55,$P$4:$P$10)+SUMIF($N$16:$N$22,$M55,$P$16:$P$22)+SUMIF($N$31:$N$33,$M55,$P$31:$P$33)+SUMIF($N$42:$N$46,$M55,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P55" s="116">
@@ -4937,7 +5215,7 @@
         </is>
       </c>
       <c r="T55" s="122">
-        <f>SUMIF($S$2:$S$47,$R55,$U$2:$U$47)</f>
+        <f>SUMIF($S$4:$S$10,$R55,$U$4:$U$10)+SUMIF($S$16:$S$22,$R55,$U$16:$U$22)+SUMIF($S$31:$S$33,$R55,$U$31:$U$33)+SUMIF($S$42:$S$46,$R55,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U55" s="116">
@@ -4966,7 +5244,7 @@
         </is>
       </c>
       <c r="E56" s="122">
-        <f>SUMIF($D$2:$D$47,$C56,$F$2:$F$47)</f>
+        <f>SUMIF($D$4:$D$10,$C56,$F$4:$F$10)+SUMIF($D$16:$D$22,$C56,$F$16:$F$22)+SUMIF($D$31:$D$33,$C56,$F$31:$F$33)+SUMIF($D$42:$D$46,$C56,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F56" s="116">
@@ -4987,7 +5265,7 @@
         </is>
       </c>
       <c r="J56" s="122">
-        <f>SUMIF($I$2:$I$47,$H56,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H56,$K$4:$K$10)+SUMIF($I$16:$I$22,$H56,$K$16:$K$22)+SUMIF($I$31:$I$33,$H56,$K$31:$K$33)+SUMIF($I$42:$I$46,$H56,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K56" s="116">
@@ -5008,7 +5286,7 @@
         </is>
       </c>
       <c r="O56" s="122">
-        <f>SUMIF($N$2:$N$47,$M56,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M56,$P$4:$P$10)+SUMIF($N$16:$N$22,$M56,$P$16:$P$22)+SUMIF($N$31:$N$33,$M56,$P$31:$P$33)+SUMIF($N$42:$N$46,$M56,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P56" s="116">
@@ -5029,7 +5307,7 @@
         </is>
       </c>
       <c r="T56" s="122">
-        <f>SUMIF($S$2:$S$47,$R56,$U$2:$U$47)</f>
+        <f>SUMIF($S$4:$S$10,$R56,$U$4:$U$10)+SUMIF($S$16:$S$22,$R56,$U$16:$U$22)+SUMIF($S$31:$S$33,$R56,$U$31:$U$33)+SUMIF($S$42:$S$46,$R56,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U56" s="116">
@@ -5058,7 +5336,7 @@
         </is>
       </c>
       <c r="E57" s="123">
-        <f>SUMIF($D$2:$D$47,$C57,$F$2:$F$47)</f>
+        <f>SUMIF($D$4:$D$10,$C57,$F$4:$F$10)+SUMIF($D$16:$D$22,$C57,$F$16:$F$22)+SUMIF($D$31:$D$33,$C57,$F$31:$F$33)+SUMIF($D$42:$D$46,$C57,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F57" s="117">
@@ -5079,7 +5357,7 @@
         </is>
       </c>
       <c r="J57" s="123">
-        <f>SUMIF($I$2:$I$47,$H57,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H57,$K$4:$K$10)+SUMIF($I$16:$I$22,$H57,$K$16:$K$22)+SUMIF($I$31:$I$33,$H57,$K$31:$K$33)+SUMIF($I$42:$I$46,$H57,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K57" s="117">
@@ -5100,7 +5378,7 @@
         </is>
       </c>
       <c r="O57" s="123">
-        <f>SUMIF($N$2:$N$47,$M57,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M57,$P$4:$P$10)+SUMIF($N$16:$N$22,$M57,$P$16:$P$22)+SUMIF($N$31:$N$33,$M57,$P$31:$P$33)+SUMIF($N$42:$N$46,$M57,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P57" s="117">
@@ -5121,7 +5399,7 @@
         </is>
       </c>
       <c r="T57" s="123">
-        <f>SUMIF($S$2:$S$47,$R57,$U$2:$U$47)</f>
+        <f>SUMIF($S$4:$S$10,$R57,$U$4:$U$10)+SUMIF($S$16:$S$22,$R57,$U$16:$U$22)+SUMIF($S$31:$S$33,$R57,$U$31:$U$33)+SUMIF($S$42:$S$46,$R57,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U57" s="117">
@@ -5153,15 +5431,15 @@
           <t>承攬工程收入</t>
         </is>
       </c>
-      <c r="E58" s="124">
-        <f>SUMIF($D$2:$D$47,$C58,$F$2:$F$47)</f>
-        <v/>
-      </c>
-      <c r="F58" s="206">
+      <c r="E58" s="216">
+        <f>SUMIF($D$4:$D$10,$C58,$F$4:$F$10)+SUMIF($D$16:$D$22,$C58,$F$16:$F$22)+SUMIF($D$31:$D$33,$C58,$F$31:$F$33)+SUMIF($D$42:$D$46,$C58,$F$42:$F$46)</f>
+        <v/>
+      </c>
+      <c r="F58" s="205">
         <f>SUM(E58:E68)</f>
         <v/>
       </c>
-      <c r="G58" s="207" t="inlineStr">
+      <c r="G58" s="206" t="inlineStr">
         <is>
           <t>本期損益</t>
         </is>
@@ -5175,14 +5453,14 @@
         </is>
       </c>
       <c r="J58" s="124">
-        <f>SUMIF($I$2:$I$47,$H58,$K$2:$K$47)</f>
-        <v/>
-      </c>
-      <c r="K58" s="206">
+        <f>SUMIF($I$4:$I$10,$H58,$K$4:$K$10)+SUMIF($I$16:$I$22,$H58,$K$16:$K$22)+SUMIF($I$31:$I$33,$H58,$K$31:$K$33)+SUMIF($I$42:$I$46,$H58,$K$42:$K$46)</f>
+        <v/>
+      </c>
+      <c r="K58" s="205">
         <f>SUM(J58:J68)</f>
         <v/>
       </c>
-      <c r="L58" s="207" t="inlineStr">
+      <c r="L58" s="206" t="inlineStr">
         <is>
           <t>本期損益</t>
         </is>
@@ -5196,14 +5474,14 @@
         </is>
       </c>
       <c r="O58" s="124">
-        <f>SUMIF($N$2:$N$47,$M58,$P$2:$P$47)</f>
-        <v/>
-      </c>
-      <c r="P58" s="206">
+        <f>SUMIF($N$4:$N$10,$M58,$P$4:$P$10)+SUMIF($N$16:$N$22,$M58,$P$16:$P$22)+SUMIF($N$31:$N$33,$M58,$P$31:$P$33)+SUMIF($N$42:$N$46,$M58,$P$42:$P$46)</f>
+        <v/>
+      </c>
+      <c r="P58" s="205">
         <f>SUM(O58:O68)</f>
         <v/>
       </c>
-      <c r="Q58" s="207" t="inlineStr">
+      <c r="Q58" s="206" t="inlineStr">
         <is>
           <t>本期損益</t>
         </is>
@@ -5217,14 +5495,14 @@
         </is>
       </c>
       <c r="T58" s="124">
-        <f>SUMIF($S$2:$S$47,$R58,$U$2:$U$47)</f>
-        <v/>
-      </c>
-      <c r="U58" s="206">
+        <f>SUMIF($S$4:$S$10,$R58,$U$4:$U$10)+SUMIF($S$16:$S$22,$R58,$U$16:$U$22)+SUMIF($S$31:$S$33,$R58,$U$31:$U$33)+SUMIF($S$42:$S$46,$R58,$U$42:$U$46)</f>
+        <v/>
+      </c>
+      <c r="U58" s="205">
         <f>SUM(T58:T68)</f>
         <v/>
       </c>
-      <c r="V58" s="207" t="inlineStr">
+      <c r="V58" s="206" t="inlineStr">
         <is>
           <t>本期損益</t>
         </is>
@@ -5245,8 +5523,8 @@
           <t>承攬工程成本</t>
         </is>
       </c>
-      <c r="E59" s="124">
-        <f>SUMIF($D$2:$D$47,$C59,$F$2:$F$47)</f>
+      <c r="E59" s="216">
+        <f>SUMIF($D$4:$D$10,$C59,$F$4:$F$10)+SUMIF($D$16:$D$22,$C59,$F$16:$F$22)+SUMIF($D$31:$D$33,$C59,$F$31:$F$33)+SUMIF($D$42:$D$46,$C59,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F59" s="201" t="n"/>
@@ -5260,39 +5538,35 @@
         </is>
       </c>
       <c r="J59" s="124">
-        <f>SUMIF($I$2:$I$47,$H59,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H59,$K$4:$K$10)+SUMIF($I$16:$I$22,$H59,$K$16:$K$22)+SUMIF($I$31:$I$33,$H59,$K$31:$K$33)+SUMIF($I$42:$I$46,$H59,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K59" s="201" t="n"/>
       <c r="L59" s="202" t="n"/>
-      <c r="M59" s="208" t="inlineStr">
-        <is>
-          <t>55110095</t>
-        </is>
-      </c>
-      <c r="N59" s="195" t="inlineStr">
-        <is>
-          <t>承攬工程成本-其他</t>
-        </is>
-      </c>
-      <c r="O59" s="203">
-        <f>SUMIF($N$2:$N$47,$M59,$P$2:$P$47)</f>
+      <c r="M59" s="138" t="n">
+        <v>55110000</v>
+      </c>
+      <c r="N59" s="103" t="inlineStr">
+        <is>
+          <t>承攬工程成本</t>
+        </is>
+      </c>
+      <c r="O59" s="124">
+        <f>SUMIF($N$4:$N$10,$M59,$P$4:$P$10)+SUMIF($N$16:$N$22,$M59,$P$16:$P$22)+SUMIF($N$31:$N$33,$M59,$P$31:$P$33)+SUMIF($N$42:$N$46,$M59,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P59" s="201" t="n"/>
       <c r="Q59" s="202" t="n"/>
-      <c r="R59" s="208" t="inlineStr">
-        <is>
-          <t>62370030</t>
-        </is>
-      </c>
-      <c r="S59" s="195" t="inlineStr">
-        <is>
-          <t>勞務費-其他</t>
-        </is>
-      </c>
-      <c r="T59" s="203">
-        <f>SUMIF($S$2:$S$47,$R59,$U$2:$U$47)</f>
+      <c r="R59" s="138" t="n">
+        <v>55110000</v>
+      </c>
+      <c r="S59" s="103" t="inlineStr">
+        <is>
+          <t>承攬工程成本</t>
+        </is>
+      </c>
+      <c r="T59" s="124">
+        <f>SUMIF($S$4:$S$10,$R59,$U$4:$U$10)+SUMIF($S$16:$S$22,$R59,$U$16:$U$22)+SUMIF($S$31:$S$33,$R59,$U$31:$U$33)+SUMIF($S$42:$S$46,$R59,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U59" s="201" t="n"/>
@@ -5305,18 +5579,10 @@
     <row r="60">
       <c r="A60" s="199" t="n"/>
       <c r="B60" s="200" t="n"/>
-      <c r="C60" s="209" t="inlineStr">
-        <is>
-          <t>55110095</t>
-        </is>
-      </c>
-      <c r="D60" s="195" t="inlineStr">
-        <is>
-          <t>承攬工程成本-其他</t>
-        </is>
-      </c>
-      <c r="E60" s="203">
-        <f>SUMIF($D$2:$D$47,$C60,$F$2:$F$47)</f>
+      <c r="C60" s="102" t="n"/>
+      <c r="D60" s="103" t="n"/>
+      <c r="E60" s="124">
+        <f>SUMIF($D$4:$D$10,$C60,$F$4:$F$10)+SUMIF($D$16:$D$22,$C60,$F$16:$F$22)+SUMIF($D$31:$D$33,$C60,$F$31:$F$33)+SUMIF($D$42:$D$46,$C60,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F60" s="201" t="n"/>
@@ -5324,7 +5590,7 @@
       <c r="H60" s="138" t="n"/>
       <c r="I60" s="103" t="n"/>
       <c r="J60" s="124">
-        <f>SUMIF($I$2:$I$47,$H60,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H60,$K$4:$K$10)+SUMIF($I$16:$I$22,$H60,$K$16:$K$22)+SUMIF($I$31:$I$33,$H60,$K$31:$K$33)+SUMIF($I$42:$I$46,$H60,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K60" s="201" t="n"/>
@@ -5340,7 +5606,7 @@
         </is>
       </c>
       <c r="O60" s="124">
-        <f>SUMIF($N$2:$N$47,$M60,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M60,$P$4:$P$10)+SUMIF($N$16:$N$22,$M60,$P$16:$P$22)+SUMIF($N$31:$N$33,$M60,$P$31:$P$33)+SUMIF($N$42:$N$46,$M60,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P60" s="201" t="n"/>
@@ -5355,8 +5621,8 @@
           <t>專案成本</t>
         </is>
       </c>
-      <c r="T60" s="124">
-        <f>SUMIF($S$2:$S$47,$R60,$U$2:$U$47)</f>
+      <c r="T60" s="216">
+        <f>SUMIF($S$4:$S$10,$R60,$U$4:$U$10)+SUMIF($S$16:$S$22,$R60,$U$16:$U$22)+SUMIF($S$31:$S$33,$R60,$U$31:$U$33)+SUMIF($S$42:$S$46,$R60,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U60" s="201" t="n"/>
@@ -5369,42 +5635,29 @@
     <row r="61">
       <c r="A61" s="199" t="n"/>
       <c r="B61" s="200" t="n"/>
-      <c r="C61" s="209" t="inlineStr">
-        <is>
-          <t>63670100</t>
-        </is>
-      </c>
-      <c r="D61" s="195" t="inlineStr">
-        <is>
-          <t>工程工務所費用-其他費用</t>
-        </is>
-      </c>
-      <c r="E61" s="203">
-        <f>SUMIF($D$2:$D$47,$C61,$F$2:$F$47)</f>
-        <v/>
-      </c>
+      <c r="C61" s="102" t="n"/>
+      <c r="D61" s="103" t="n"/>
+      <c r="E61" s="124" t="n"/>
       <c r="F61" s="201" t="n"/>
       <c r="G61" s="202" t="n"/>
       <c r="H61" s="102" t="n"/>
       <c r="I61" s="103" t="n"/>
       <c r="J61" s="124">
-        <f>SUMIF($I$2:$I$47,$H61,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H61,$K$4:$K$10)+SUMIF($I$16:$I$22,$H61,$K$16:$K$22)+SUMIF($I$31:$I$33,$H61,$K$31:$K$33)+SUMIF($I$42:$I$46,$H61,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K61" s="201" t="n"/>
       <c r="L61" s="202" t="n"/>
-      <c r="M61" s="208" t="inlineStr">
-        <is>
-          <t>63670100</t>
-        </is>
-      </c>
-      <c r="N61" s="195" t="inlineStr">
-        <is>
-          <t>工程工務所費用-其他費用</t>
-        </is>
-      </c>
-      <c r="O61" s="203">
-        <f>SUMIF($N$2:$N$47,$M61,$P$2:$P$47)</f>
+      <c r="M61" s="138" t="n">
+        <v>55110098</v>
+      </c>
+      <c r="N61" s="103" t="inlineStr">
+        <is>
+          <t>承攬工程成本-非人事</t>
+        </is>
+      </c>
+      <c r="O61" s="124">
+        <f>SUMIF($N$4:$N$10,$M61,$P$4:$P$10)+SUMIF($N$16:$N$22,$M61,$P$16:$P$22)+SUMIF($N$31:$N$33,$M61,$P$31:$P$33)+SUMIF($N$42:$N$46,$M61,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P61" s="201" t="n"/>
@@ -5418,7 +5671,7 @@
         </is>
       </c>
       <c r="T61" s="124">
-        <f>SUMIF($S$2:$S$47,$R61,$U$2:$U$47)</f>
+        <f>SUMIF($S$4:$S$10,$R61,$U$4:$U$10)+SUMIF($S$16:$S$22,$R61,$U$16:$U$22)+SUMIF($S$31:$S$33,$R61,$U$31:$U$33)+SUMIF($S$42:$S$46,$R61,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U61" s="201" t="n"/>
@@ -5442,7 +5695,7 @@
         </is>
       </c>
       <c r="E62" s="124">
-        <f>SUMIF($D$2:$D$47,$C62,$F$2:$F$47)</f>
+        <f>SUMIF($D$4:$D$10,$C62,$F$4:$F$10)+SUMIF($D$16:$D$22,$C62,$F$16:$F$22)+SUMIF($D$31:$D$33,$C62,$F$31:$F$33)+SUMIF($D$42:$D$46,$C62,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F62" s="201" t="n"/>
@@ -5458,7 +5711,7 @@
         </is>
       </c>
       <c r="J62" s="124">
-        <f>SUMIF($I$2:$I$47,$H62,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H62,$K$4:$K$10)+SUMIF($I$16:$I$22,$H62,$K$16:$K$22)+SUMIF($I$31:$I$33,$H62,$K$31:$K$33)+SUMIF($I$42:$I$46,$H62,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K62" s="201" t="n"/>
@@ -5473,8 +5726,8 @@
           <t>勞務收入-內部計價</t>
         </is>
       </c>
-      <c r="O62" s="203">
-        <f>SUMIF($N$2:$N$47,$M62,$P$2:$P$47)</f>
+      <c r="O62" s="124">
+        <f>SUMIF($N$4:$N$10,$M62,$P$4:$P$10)+SUMIF($N$16:$N$22,$M62,$P$16:$P$22)+SUMIF($N$31:$N$33,$M62,$P$31:$P$33)+SUMIF($N$42:$N$46,$M62,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P62" s="201" t="n"/>
@@ -5489,8 +5742,8 @@
           <t>勞務收入-內部計價</t>
         </is>
       </c>
-      <c r="T62" s="203">
-        <f>SUMIF($S$2:$S$47,$R62,$U$2:$U$47)</f>
+      <c r="T62" s="124">
+        <f>SUMIF($S$4:$S$10,$R62,$U$4:$U$10)+SUMIF($S$16:$S$22,$R62,$U$16:$U$22)+SUMIF($S$31:$S$33,$R62,$U$31:$U$33)+SUMIF($S$42:$S$46,$R62,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U62" s="201" t="n"/>
@@ -5506,7 +5759,7 @@
       <c r="C63" s="102" t="n"/>
       <c r="D63" s="103" t="n"/>
       <c r="E63" s="124">
-        <f>SUMIF($D$2:$D$47,$C63,$F$2:$F$47)</f>
+        <f>SUMIF($D$4:$D$10,$C63,$F$4:$F$10)+SUMIF($D$16:$D$22,$C63,$F$16:$F$22)+SUMIF($D$31:$D$33,$C63,$F$31:$F$33)+SUMIF($D$42:$D$46,$C63,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F63" s="201" t="n"/>
@@ -5514,7 +5767,7 @@
       <c r="H63" s="138" t="n"/>
       <c r="I63" s="103" t="n"/>
       <c r="J63" s="124">
-        <f>SUMIF($I$2:$I$47,$H63,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H63,$K$4:$K$10)+SUMIF($I$16:$I$22,$H63,$K$16:$K$22)+SUMIF($I$31:$I$33,$H63,$K$31:$K$33)+SUMIF($I$42:$I$46,$H63,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K63" s="201" t="n"/>
@@ -5530,7 +5783,7 @@
         </is>
       </c>
       <c r="O63" s="124">
-        <f>SUMIF($N$2:$N$47,$M63,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M63,$P$4:$P$10)+SUMIF($N$16:$N$22,$M63,$P$16:$P$22)+SUMIF($N$31:$N$33,$M63,$P$31:$P$33)+SUMIF($N$42:$N$46,$M63,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P63" s="201" t="n"/>
@@ -5546,7 +5799,7 @@
         </is>
       </c>
       <c r="T63" s="124">
-        <f>SUMIF($S$2:$S$47,$R63,$U$2:$U$47)</f>
+        <f>SUMIF($S$4:$S$10,$R63,$U$4:$U$10)+SUMIF($S$16:$S$22,$R63,$U$16:$U$22)+SUMIF($S$31:$S$33,$R63,$U$31:$U$33)+SUMIF($S$42:$S$46,$R63,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U63" s="201" t="n"/>
@@ -5567,7 +5820,7 @@
       <c r="H64" s="102" t="n"/>
       <c r="I64" s="103" t="n"/>
       <c r="J64" s="124">
-        <f>SUMIF($I$2:$I$47,$H64,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H64,$K$4:$K$10)+SUMIF($I$16:$I$22,$H64,$K$16:$K$22)+SUMIF($I$31:$I$33,$H64,$K$31:$K$33)+SUMIF($I$42:$I$46,$H64,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K64" s="201" t="n"/>
@@ -5581,7 +5834,7 @@
         </is>
       </c>
       <c r="O64" s="124">
-        <f>SUMIF($N$2:$N$47,$M64,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M64,$P$4:$P$10)+SUMIF($N$16:$N$22,$M64,$P$16:$P$22)+SUMIF($N$31:$N$33,$M64,$P$31:$P$33)+SUMIF($N$42:$N$46,$M64,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P64" s="201" t="n"/>
@@ -5594,8 +5847,8 @@
           <t>人事分攤</t>
         </is>
       </c>
-      <c r="T64" s="124">
-        <f>SUMIF($S$2:$S$47,$R64,$U$2:$U$47)</f>
+      <c r="T64" s="216">
+        <f>SUMIF($S$4:$S$10,$R64,$U$4:$U$10)+SUMIF($S$16:$S$22,$R64,$U$16:$U$22)+SUMIF($S$31:$S$33,$R64,$U$31:$U$33)+SUMIF($S$42:$S$46,$R64,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U64" s="201" t="n"/>
@@ -5616,7 +5869,7 @@
       <c r="H65" s="102" t="n"/>
       <c r="I65" s="103" t="n"/>
       <c r="J65" s="124">
-        <f>SUMIF($I$2:$I$47,$H65,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H65,$K$4:$K$10)+SUMIF($I$16:$I$22,$H65,$K$16:$K$22)+SUMIF($I$31:$I$33,$H65,$K$31:$K$33)+SUMIF($I$42:$I$46,$H65,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K65" s="201" t="n"/>
@@ -5630,7 +5883,7 @@
         </is>
       </c>
       <c r="O65" s="124">
-        <f>SUMIF($N$2:$N$47,$M65,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M65,$P$4:$P$10)+SUMIF($N$16:$N$22,$M65,$P$16:$P$22)+SUMIF($N$31:$N$33,$M65,$P$31:$P$33)+SUMIF($N$42:$N$46,$M65,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P65" s="201" t="n"/>
@@ -5643,8 +5896,8 @@
           <t>勞務費-收回投標費</t>
         </is>
       </c>
-      <c r="T65" s="203">
-        <f>SUMIF($S$2:$S$47,$R65,$U$2:$U$47)</f>
+      <c r="T65" s="124">
+        <f>SUMIF($S$4:$S$10,$R65,$U$4:$U$10)+SUMIF($S$16:$S$22,$R65,$U$16:$U$22)+SUMIF($S$31:$S$33,$R65,$U$31:$U$33)+SUMIF($S$42:$S$46,$R65,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U65" s="201" t="n"/>
@@ -5660,7 +5913,7 @@
       <c r="C66" s="102" t="n"/>
       <c r="D66" s="103" t="n"/>
       <c r="E66" s="124">
-        <f>SUMIF($D$2:$D$47,$C66,$F$2:$F$47)</f>
+        <f>SUMIF($D$4:$D$10,$C66,$F$4:$F$10)+SUMIF($D$16:$D$22,$C66,$F$16:$F$22)+SUMIF($D$31:$D$33,$C66,$F$31:$F$33)+SUMIF($D$42:$D$46,$C66,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F66" s="201" t="n"/>
@@ -5668,7 +5921,7 @@
       <c r="H66" s="138" t="n"/>
       <c r="I66" s="103" t="n"/>
       <c r="J66" s="124">
-        <f>SUMIF($I$2:$I$47,$H66,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H66,$K$4:$K$10)+SUMIF($I$16:$I$22,$H66,$K$16:$K$22)+SUMIF($I$31:$I$33,$H66,$K$31:$K$33)+SUMIF($I$42:$I$46,$H66,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K66" s="201" t="n"/>
@@ -5682,7 +5935,7 @@
         </is>
       </c>
       <c r="O66" s="124">
-        <f>SUMIF($N$2:$N$47,$M66,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M66,$P$4:$P$10)+SUMIF($N$16:$N$22,$M66,$P$16:$P$22)+SUMIF($N$31:$N$33,$M66,$P$31:$P$33)+SUMIF($N$42:$N$46,$M66,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P66" s="201" t="n"/>
@@ -5695,8 +5948,8 @@
           <t>電腦out charge</t>
         </is>
       </c>
-      <c r="T66" s="124">
-        <f>SUMIF($S$2:$S$47,$R66,$U$2:$U$47)</f>
+      <c r="T66" s="216">
+        <f>SUMIF($S$4:$S$10,$R66,$U$4:$U$10)+SUMIF($S$16:$S$22,$R66,$U$16:$U$22)+SUMIF($S$31:$S$33,$R66,$U$31:$U$33)+SUMIF($S$42:$S$46,$R66,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U66" s="201" t="n"/>
@@ -5720,7 +5973,7 @@
         </is>
       </c>
       <c r="E67" s="124">
-        <f>SUMIF($D$2:$D$47,$C67,$F$2:$F$47)</f>
+        <f>SUMIF($D$4:$D$10,$C67,$F$4:$F$10)+SUMIF($D$16:$D$22,$C67,$F$16:$F$22)+SUMIF($D$31:$D$33,$C67,$F$31:$F$33)+SUMIF($D$42:$D$46,$C67,$F$42:$F$46)</f>
         <v/>
       </c>
       <c r="F67" s="201" t="n"/>
@@ -5736,7 +5989,7 @@
         </is>
       </c>
       <c r="J67" s="124">
-        <f>SUMIF($I$2:$I$47,$H67,$K$2:$K$47)</f>
+        <f>SUMIF($I$4:$I$10,$H67,$K$4:$K$10)+SUMIF($I$16:$I$22,$H67,$K$16:$K$22)+SUMIF($I$31:$I$33,$H67,$K$31:$K$33)+SUMIF($I$42:$I$46,$H67,$K$42:$K$46)</f>
         <v/>
       </c>
       <c r="K67" s="201" t="n"/>
@@ -5752,7 +6005,7 @@
         </is>
       </c>
       <c r="O67" s="124">
-        <f>SUMIF($N$2:$N$47,$M67,$P$2:$P$47)</f>
+        <f>SUMIF($N$4:$N$10,$M67,$P$4:$P$10)+SUMIF($N$16:$N$22,$M67,$P$16:$P$22)+SUMIF($N$31:$N$33,$M67,$P$31:$P$33)+SUMIF($N$42:$N$46,$M67,$P$42:$P$46)</f>
         <v/>
       </c>
       <c r="P67" s="201" t="n"/>
@@ -5768,7 +6021,7 @@
         </is>
       </c>
       <c r="T67" s="124">
-        <f>SUMIF($S$2:$S$47,$R67,$U$2:$U$47)</f>
+        <f>SUMIF($S$4:$S$10,$R67,$U$4:$U$10)+SUMIF($S$16:$S$22,$R67,$U$16:$U$22)+SUMIF($S$31:$S$33,$R67,$U$31:$U$33)+SUMIF($S$42:$S$46,$R67,$U$42:$U$46)</f>
         <v/>
       </c>
       <c r="U67" s="201" t="n"/>
@@ -5779,8 +6032,8 @@
       <c r="Z67" s="79" t="n"/>
     </row>
     <row r="68" ht="16.2" customHeight="1" s="186" thickBot="1">
-      <c r="A68" s="210" t="n"/>
-      <c r="B68" s="211" t="n"/>
+      <c r="A68" s="207" t="n"/>
+      <c r="B68" s="208" t="n"/>
       <c r="C68" s="107" t="n">
         <v>63810030</v>
       </c>
@@ -5790,11 +6043,11 @@
         </is>
       </c>
       <c r="E68" s="125">
-        <f>SUMIF($D$2:$D$47,$C68,$F$2:$F$47)</f>
-        <v/>
-      </c>
-      <c r="F68" s="212" t="n"/>
-      <c r="G68" s="213" t="n"/>
+        <f>SUMIF($D$4:$D$10,$C68,$F$4:$F$10)+SUMIF($D$16:$D$22,$C68,$F$16:$F$22)+SUMIF($D$31:$D$33,$C68,$F$31:$F$33)+SUMIF($D$42:$D$46,$C68,$F$42:$F$46)</f>
+        <v/>
+      </c>
+      <c r="F68" s="209" t="n"/>
+      <c r="G68" s="210" t="n"/>
       <c r="H68" s="139" t="n">
         <v>63810030</v>
       </c>
@@ -5804,11 +6057,11 @@
         </is>
       </c>
       <c r="J68" s="125">
-        <f>SUMIF($I$2:$I$47,$H68,$K$2:$K$47)</f>
-        <v/>
-      </c>
-      <c r="K68" s="212" t="n"/>
-      <c r="L68" s="213" t="n"/>
+        <f>SUMIF($I$4:$I$10,$H68,$K$4:$K$10)+SUMIF($I$16:$I$22,$H68,$K$16:$K$22)+SUMIF($I$31:$I$33,$H68,$K$31:$K$33)+SUMIF($I$42:$I$46,$H68,$K$42:$K$46)</f>
+        <v/>
+      </c>
+      <c r="K68" s="209" t="n"/>
+      <c r="L68" s="210" t="n"/>
       <c r="M68" s="139" t="n">
         <v>63810030</v>
       </c>
@@ -5818,11 +6071,11 @@
         </is>
       </c>
       <c r="O68" s="125">
-        <f>SUMIF($N$2:$N$47,$M68,$P$2:$P$47)</f>
-        <v/>
-      </c>
-      <c r="P68" s="212" t="n"/>
-      <c r="Q68" s="213" t="n"/>
+        <f>SUMIF($N$4:$N$10,$M68,$P$4:$P$10)+SUMIF($N$16:$N$22,$M68,$P$16:$P$22)+SUMIF($N$31:$N$33,$M68,$P$31:$P$33)+SUMIF($N$42:$N$46,$M68,$P$42:$P$46)</f>
+        <v/>
+      </c>
+      <c r="P68" s="209" t="n"/>
+      <c r="Q68" s="210" t="n"/>
       <c r="R68" s="139" t="n">
         <v>63810030</v>
       </c>
@@ -5832,11 +6085,11 @@
         </is>
       </c>
       <c r="T68" s="125">
-        <f>SUMIF($S$2:$S$47,$R68,$U$2:$U$47)</f>
-        <v/>
-      </c>
-      <c r="U68" s="212" t="n"/>
-      <c r="V68" s="213" t="n"/>
+        <f>SUMIF($S$4:$S$10,$R68,$U$4:$U$10)+SUMIF($S$16:$S$22,$R68,$U$16:$U$22)+SUMIF($S$31:$S$33,$R68,$U$31:$U$33)+SUMIF($S$42:$S$46,$R68,$U$42:$U$46)</f>
+        <v/>
+      </c>
+      <c r="U68" s="209" t="n"/>
+      <c r="V68" s="210" t="n"/>
       <c r="W68" s="79" t="n"/>
       <c r="X68" s="79" t="n"/>
       <c r="Y68" s="79" t="n"/>
@@ -5851,37 +6104,37 @@
           <t>check</t>
         </is>
       </c>
-      <c r="E69" s="214">
+      <c r="E69" s="211">
         <f>SUM(E50:E68)</f>
         <v/>
       </c>
-      <c r="F69" s="214">
+      <c r="F69" s="211">
         <f>SUM(F50:F68)</f>
         <v/>
       </c>
       <c r="G69" s="28" t="n"/>
       <c r="H69" s="79" t="n"/>
-      <c r="J69" s="214">
+      <c r="J69" s="211">
         <f>SUM(J50:J68)</f>
         <v/>
       </c>
-      <c r="K69" s="214">
+      <c r="K69" s="211">
         <f>SUM(K50:K68)</f>
         <v/>
       </c>
-      <c r="O69" s="214">
+      <c r="O69" s="211">
         <f>SUM(O50:O68)</f>
         <v/>
       </c>
-      <c r="P69" s="214">
+      <c r="P69" s="211">
         <f>SUM(P50:P68)</f>
         <v/>
       </c>
-      <c r="T69" s="214">
+      <c r="T69" s="211">
         <f>SUM(T50:T68)</f>
         <v/>
       </c>
-      <c r="U69" s="214">
+      <c r="U69" s="211">
         <f>SUM(U50:U68)</f>
         <v/>
       </c>
@@ -6036,10 +6289,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:S47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" style="186" min="1" max="1"/>
+    <col width="46" customWidth="1" style="186" min="1" max="1"/>
     <col width="14" customWidth="1" style="186" min="2" max="2"/>
     <col width="14" customWidth="1" style="186" min="3" max="3"/>
     <col width="14" customWidth="1" style="186" min="4" max="4"/>
@@ -6047,14 +6300,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="215" t="inlineStr">
+      <c r="A1" s="212" t="inlineStr">
         <is>
           <t>A. 每筆分錄借貸差（應為0）</t>
         </is>
       </c>
-      <c r="G1" s="215" t="inlineStr">
-        <is>
-          <t>輔助：主表每列科目類別與金額</t>
+      <c r="G1" s="212" t="inlineStr">
+        <is>
+          <t>輔助：主表每列（非BIM列記為空）</t>
         </is>
       </c>
     </row>
@@ -6064,22 +6317,22 @@
           <t>分錄</t>
         </is>
       </c>
-      <c r="B2" s="215" t="inlineStr">
+      <c r="B2" s="212" t="inlineStr">
         <is>
           <t>內案POC</t>
         </is>
       </c>
-      <c r="C2" s="215" t="inlineStr">
+      <c r="C2" s="212" t="inlineStr">
         <is>
           <t>外案POC</t>
         </is>
       </c>
-      <c r="D2" s="215" t="inlineStr">
+      <c r="D2" s="212" t="inlineStr">
         <is>
           <t>雜項</t>
         </is>
       </c>
-      <c r="E2" s="215" t="inlineStr">
+      <c r="E2" s="212" t="inlineStr">
         <is>
           <t>備標</t>
         </is>
@@ -6091,60 +6344,80 @@
           <t>1 費用入帳（第4-6列）</t>
         </is>
       </c>
-      <c r="B3" s="216">
+      <c r="B3" s="213">
         <f>ROUND(SUM('工作表1'!F4:F6),6)</f>
         <v/>
       </c>
-      <c r="C3" s="216">
+      <c r="C3" s="213">
         <f>ROUND(SUM('工作表1'!K4:K6),6)</f>
         <v/>
       </c>
-      <c r="D3" s="216">
+      <c r="D3" s="213">
         <f>ROUND(SUM('工作表1'!P4:P6),6)</f>
         <v/>
       </c>
-      <c r="E3" s="216">
+      <c r="E3" s="213">
         <f>ROUND(SUM('工作表1'!U4:U6),6)</f>
         <v/>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>內案類別</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>內案金額</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>外案類別</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>外案金額</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t>內案POC類別</t>
+        </is>
+      </c>
+      <c r="I3" s="0" t="inlineStr">
+        <is>
+          <t>內案POC金額</t>
+        </is>
+      </c>
+      <c r="J3" s="0" t="inlineStr">
+        <is>
+          <t>內案POC未入總結</t>
+        </is>
+      </c>
+      <c r="K3" s="0" t="inlineStr">
+        <is>
+          <t>外案POC類別</t>
+        </is>
+      </c>
+      <c r="L3" s="0" t="inlineStr">
+        <is>
+          <t>外案POC金額</t>
+        </is>
+      </c>
+      <c r="M3" s="0" t="inlineStr">
+        <is>
+          <t>外案POC未入總結</t>
+        </is>
+      </c>
+      <c r="N3" s="0" t="inlineStr">
         <is>
           <t>雜項類別</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" s="0" t="inlineStr">
         <is>
           <t>雜項金額</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" s="0" t="inlineStr">
+        <is>
+          <t>雜項未入總結</t>
+        </is>
+      </c>
+      <c r="Q3" s="0" t="inlineStr">
         <is>
           <t>備標類別</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="R3" s="0" t="inlineStr">
         <is>
           <t>備標金額</t>
+        </is>
+      </c>
+      <c r="S3" s="0" t="inlineStr">
+        <is>
+          <t>備標未入總結</t>
         </is>
       </c>
     </row>
@@ -6154,57 +6427,68 @@
           <t>2 費用轉列成本（第8-10列）</t>
         </is>
       </c>
-      <c r="B4" s="216">
+      <c r="B4" s="213">
         <f>ROUND(SUM('工作表1'!F8:F10),6)</f>
         <v/>
       </c>
-      <c r="C4" s="216">
+      <c r="C4" s="213">
         <f>ROUND(SUM('工作表1'!K8:K10),6)</f>
         <v/>
       </c>
-      <c r="D4" s="216">
+      <c r="D4" s="213">
         <f>ROUND(SUM('工作表1'!P8:P10),6)</f>
         <v/>
       </c>
-      <c r="E4" s="216">
+      <c r="E4" s="213">
         <f>ROUND(SUM('工作表1'!U8:U10),6)</f>
         <v/>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>主表列號4起</t>
-        </is>
-      </c>
-      <c r="H4">
+      <c r="H4" s="0">
         <f>IF('工作表1'!D4="","",LEFT('工作表1'!D4,1))</f>
         <v/>
       </c>
-      <c r="I4">
+      <c r="I4" s="0">
         <f>IF(ISNUMBER('工作表1'!F4),'工作表1'!F4,0)</f>
         <v/>
       </c>
-      <c r="J4">
+      <c r="J4" s="0">
+        <f>IF('工作表1'!D4="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D4)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K4" s="0">
         <f>IF('工作表1'!I4="","",LEFT('工作表1'!I4,1))</f>
         <v/>
       </c>
-      <c r="K4">
+      <c r="L4" s="0">
         <f>IF(ISNUMBER('工作表1'!K4),'工作表1'!K4,0)</f>
         <v/>
       </c>
-      <c r="L4">
+      <c r="M4" s="0">
+        <f>IF('工作表1'!I4="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I4)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N4" s="0">
         <f>IF('工作表1'!N4="","",LEFT('工作表1'!N4,1))</f>
         <v/>
       </c>
-      <c r="M4">
+      <c r="O4" s="0">
         <f>IF(ISNUMBER('工作表1'!P4),'工作表1'!P4,0)</f>
         <v/>
       </c>
-      <c r="N4">
+      <c r="P4" s="0">
+        <f>IF('工作表1'!N4="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N4)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q4" s="0">
         <f>IF('工作表1'!S4="","",LEFT('工作表1'!S4,1))</f>
         <v/>
       </c>
-      <c r="O4">
+      <c r="R4" s="0">
         <f>IF(ISNUMBER('工作表1'!U4),'工作表1'!U4,0)</f>
+        <v/>
+      </c>
+      <c r="S4" s="0">
+        <f>IF('工作表1'!S4="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S4)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -6214,52 +6498,68 @@
           <t>2 ELIA(備標)（第12-15列）</t>
         </is>
       </c>
-      <c r="B5" s="216">
+      <c r="B5" s="213">
         <f>ROUND(SUM('工作表1'!F12:F15),6)</f>
         <v/>
       </c>
-      <c r="C5" s="216">
+      <c r="C5" s="213">
         <f>ROUND(SUM('工作表1'!K12:K15),6)</f>
         <v/>
       </c>
-      <c r="D5" s="216">
+      <c r="D5" s="213">
         <f>ROUND(SUM('工作表1'!P12:P15),6)</f>
         <v/>
       </c>
-      <c r="E5" s="216">
+      <c r="E5" s="213">
         <f>ROUND(SUM('工作表1'!U12:U15),6)</f>
         <v/>
       </c>
-      <c r="H5">
+      <c r="H5" s="0">
         <f>IF('工作表1'!D5="","",LEFT('工作表1'!D5,1))</f>
         <v/>
       </c>
-      <c r="I5">
+      <c r="I5" s="0">
         <f>IF(ISNUMBER('工作表1'!F5),'工作表1'!F5,0)</f>
         <v/>
       </c>
-      <c r="J5">
+      <c r="J5" s="0">
+        <f>IF('工作表1'!D5="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D5)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K5" s="0">
         <f>IF('工作表1'!I5="","",LEFT('工作表1'!I5,1))</f>
         <v/>
       </c>
-      <c r="K5">
+      <c r="L5" s="0">
         <f>IF(ISNUMBER('工作表1'!K5),'工作表1'!K5,0)</f>
         <v/>
       </c>
-      <c r="L5">
+      <c r="M5" s="0">
+        <f>IF('工作表1'!I5="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I5)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N5" s="0">
         <f>IF('工作表1'!N5="","",LEFT('工作表1'!N5,1))</f>
         <v/>
       </c>
-      <c r="M5">
+      <c r="O5" s="0">
         <f>IF(ISNUMBER('工作表1'!P5),'工作表1'!P5,0)</f>
         <v/>
       </c>
-      <c r="N5">
+      <c r="P5" s="0">
+        <f>IF('工作表1'!N5="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N5)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q5" s="0">
         <f>IF('工作表1'!S5="","",LEFT('工作表1'!S5,1))</f>
         <v/>
       </c>
-      <c r="O5">
+      <c r="R5" s="0">
         <f>IF(ISNUMBER('工作表1'!U5),'工作表1'!U5,0)</f>
+        <v/>
+      </c>
+      <c r="S5" s="0">
+        <f>IF('工作表1'!S5="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S5)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -6269,52 +6569,68 @@
           <t>3 月底結轉在建（第16-17列）</t>
         </is>
       </c>
-      <c r="B6" s="216">
+      <c r="B6" s="213">
         <f>ROUND(SUM('工作表1'!F16:F17),6)</f>
         <v/>
       </c>
-      <c r="C6" s="216">
+      <c r="C6" s="213">
         <f>ROUND(SUM('工作表1'!K16:K17),6)</f>
         <v/>
       </c>
-      <c r="D6" s="216">
+      <c r="D6" s="213">
         <f>ROUND(SUM('工作表1'!P16:P17),6)</f>
         <v/>
       </c>
-      <c r="E6" s="216">
+      <c r="E6" s="213">
         <f>ROUND(SUM('工作表1'!U16:U17),6)</f>
         <v/>
       </c>
-      <c r="H6">
+      <c r="H6" s="0">
         <f>IF('工作表1'!D6="","",LEFT('工作表1'!D6,1))</f>
         <v/>
       </c>
-      <c r="I6">
+      <c r="I6" s="0">
         <f>IF(ISNUMBER('工作表1'!F6),'工作表1'!F6,0)</f>
         <v/>
       </c>
-      <c r="J6">
+      <c r="J6" s="0">
+        <f>IF('工作表1'!D6="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D6)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K6" s="0">
         <f>IF('工作表1'!I6="","",LEFT('工作表1'!I6,1))</f>
         <v/>
       </c>
-      <c r="K6">
+      <c r="L6" s="0">
         <f>IF(ISNUMBER('工作表1'!K6),'工作表1'!K6,0)</f>
         <v/>
       </c>
-      <c r="L6">
+      <c r="M6" s="0">
+        <f>IF('工作表1'!I6="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I6)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N6" s="0">
         <f>IF('工作表1'!N6="","",LEFT('工作表1'!N6,1))</f>
         <v/>
       </c>
-      <c r="M6">
+      <c r="O6" s="0">
         <f>IF(ISNUMBER('工作表1'!P6),'工作表1'!P6,0)</f>
         <v/>
       </c>
-      <c r="N6">
+      <c r="P6" s="0">
+        <f>IF('工作表1'!N6="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N6)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q6" s="0">
         <f>IF('工作表1'!S6="","",LEFT('工作表1'!S6,1))</f>
         <v/>
       </c>
-      <c r="O6">
+      <c r="R6" s="0">
         <f>IF(ISNUMBER('工作表1'!U6),'工作表1'!U6,0)</f>
+        <v/>
+      </c>
+      <c r="S6" s="0">
+        <f>IF('工作表1'!S6="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S6)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -6324,52 +6640,68 @@
           <t>4 完工百分比認列（第20-22列）</t>
         </is>
       </c>
-      <c r="B7" s="216">
+      <c r="B7" s="213">
         <f>ROUND(SUM('工作表1'!F20:F22),6)</f>
         <v/>
       </c>
-      <c r="C7" s="216">
+      <c r="C7" s="213">
         <f>ROUND(SUM('工作表1'!K20:K22),6)</f>
         <v/>
       </c>
-      <c r="D7" s="216">
+      <c r="D7" s="213">
         <f>ROUND(SUM('工作表1'!P20:P22),6)</f>
         <v/>
       </c>
-      <c r="E7" s="216">
+      <c r="E7" s="213">
         <f>ROUND(SUM('工作表1'!U20:U22),6)</f>
         <v/>
       </c>
-      <c r="H7">
+      <c r="H7" s="0">
         <f>IF('工作表1'!D7="","",LEFT('工作表1'!D7,1))</f>
         <v/>
       </c>
-      <c r="I7">
+      <c r="I7" s="0">
         <f>IF(ISNUMBER('工作表1'!F7),'工作表1'!F7,0)</f>
         <v/>
       </c>
-      <c r="J7">
+      <c r="J7" s="0">
+        <f>IF('工作表1'!D7="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D7)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K7" s="0">
         <f>IF('工作表1'!I7="","",LEFT('工作表1'!I7,1))</f>
         <v/>
       </c>
-      <c r="K7">
+      <c r="L7" s="0">
         <f>IF(ISNUMBER('工作表1'!K7),'工作表1'!K7,0)</f>
         <v/>
       </c>
-      <c r="L7">
+      <c r="M7" s="0">
+        <f>IF('工作表1'!I7="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I7)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N7" s="0">
         <f>IF('工作表1'!N7="","",LEFT('工作表1'!N7,1))</f>
         <v/>
       </c>
-      <c r="M7">
+      <c r="O7" s="0">
         <f>IF(ISNUMBER('工作表1'!P7),'工作表1'!P7,0)</f>
         <v/>
       </c>
-      <c r="N7">
+      <c r="P7" s="0">
+        <f>IF('工作表1'!N7="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N7)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q7" s="0">
         <f>IF('工作表1'!S7="","",LEFT('工作表1'!S7,1))</f>
         <v/>
       </c>
-      <c r="O7">
+      <c r="R7" s="0">
         <f>IF(ISNUMBER('工作表1'!U7),'工作表1'!U7,0)</f>
+        <v/>
+      </c>
+      <c r="S7" s="0">
+        <f>IF('工作表1'!S7="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S7)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -6379,52 +6711,68 @@
           <t>4 ELIA（第24-26列）</t>
         </is>
       </c>
-      <c r="B8" s="216">
+      <c r="B8" s="213">
         <f>ROUND(SUM('工作表1'!F24:F26),6)</f>
         <v/>
       </c>
-      <c r="C8" s="216">
+      <c r="C8" s="213">
         <f>ROUND(SUM('工作表1'!K24:K26),6)</f>
         <v/>
       </c>
-      <c r="D8" s="216">
+      <c r="D8" s="213">
         <f>ROUND(SUM('工作表1'!P24:P26),6)</f>
         <v/>
       </c>
-      <c r="E8" s="216">
+      <c r="E8" s="213">
         <f>ROUND(SUM('工作表1'!U24:U26),6)</f>
         <v/>
       </c>
-      <c r="H8">
+      <c r="H8" s="0">
         <f>IF('工作表1'!D8="","",LEFT('工作表1'!D8,1))</f>
         <v/>
       </c>
-      <c r="I8">
+      <c r="I8" s="0">
         <f>IF(ISNUMBER('工作表1'!F8),'工作表1'!F8,0)</f>
         <v/>
       </c>
-      <c r="J8">
+      <c r="J8" s="0">
+        <f>IF('工作表1'!D8="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D8)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K8" s="0">
         <f>IF('工作表1'!I8="","",LEFT('工作表1'!I8,1))</f>
         <v/>
       </c>
-      <c r="K8">
+      <c r="L8" s="0">
         <f>IF(ISNUMBER('工作表1'!K8),'工作表1'!K8,0)</f>
         <v/>
       </c>
-      <c r="L8">
+      <c r="M8" s="0">
+        <f>IF('工作表1'!I8="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I8)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N8" s="0">
         <f>IF('工作表1'!N8="","",LEFT('工作表1'!N8,1))</f>
         <v/>
       </c>
-      <c r="M8">
+      <c r="O8" s="0">
         <f>IF(ISNUMBER('工作表1'!P8),'工作表1'!P8,0)</f>
         <v/>
       </c>
-      <c r="N8">
+      <c r="P8" s="0">
+        <f>IF('工作表1'!N8="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N8)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q8" s="0">
         <f>IF('工作表1'!S8="","",LEFT('工作表1'!S8,1))</f>
         <v/>
       </c>
-      <c r="O8">
+      <c r="R8" s="0">
         <f>IF(ISNUMBER('工作表1'!U8),'工作表1'!U8,0)</f>
+        <v/>
+      </c>
+      <c r="S8" s="0">
+        <f>IF('工作表1'!S8="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S8)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -6434,52 +6782,68 @@
           <t>5 開立發票（第31-33列）</t>
         </is>
       </c>
-      <c r="B9" s="216">
+      <c r="B9" s="213">
         <f>ROUND(SUM('工作表1'!F31:F33),6)</f>
         <v/>
       </c>
-      <c r="C9" s="216">
+      <c r="C9" s="213">
         <f>ROUND(SUM('工作表1'!K31:K33),6)</f>
         <v/>
       </c>
-      <c r="D9" s="216">
+      <c r="D9" s="213">
         <f>ROUND(SUM('工作表1'!P31:P33),6)</f>
         <v/>
       </c>
-      <c r="E9" s="216">
+      <c r="E9" s="213">
         <f>ROUND(SUM('工作表1'!U31:U33),6)</f>
         <v/>
       </c>
-      <c r="H9">
+      <c r="H9" s="0">
         <f>IF('工作表1'!D9="","",LEFT('工作表1'!D9,1))</f>
         <v/>
       </c>
-      <c r="I9">
+      <c r="I9" s="0">
         <f>IF(ISNUMBER('工作表1'!F9),'工作表1'!F9,0)</f>
         <v/>
       </c>
-      <c r="J9">
+      <c r="J9" s="0">
+        <f>IF('工作表1'!D9="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D9)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K9" s="0">
         <f>IF('工作表1'!I9="","",LEFT('工作表1'!I9,1))</f>
         <v/>
       </c>
-      <c r="K9">
+      <c r="L9" s="0">
         <f>IF(ISNUMBER('工作表1'!K9),'工作表1'!K9,0)</f>
         <v/>
       </c>
-      <c r="L9">
+      <c r="M9" s="0">
+        <f>IF('工作表1'!I9="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I9)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N9" s="0">
         <f>IF('工作表1'!N9="","",LEFT('工作表1'!N9,1))</f>
         <v/>
       </c>
-      <c r="M9">
+      <c r="O9" s="0">
         <f>IF(ISNUMBER('工作表1'!P9),'工作表1'!P9,0)</f>
         <v/>
       </c>
-      <c r="N9">
+      <c r="P9" s="0">
+        <f>IF('工作表1'!N9="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N9)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q9" s="0">
         <f>IF('工作表1'!S9="","",LEFT('工作表1'!S9,1))</f>
         <v/>
       </c>
-      <c r="O9">
+      <c r="R9" s="0">
         <f>IF(ISNUMBER('工作表1'!U9),'工作表1'!U9,0)</f>
+        <v/>
+      </c>
+      <c r="S9" s="0">
+        <f>IF('工作表1'!S9="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S9)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -6489,52 +6853,68 @@
           <t>5 TBU認列成本（第35-36列）</t>
         </is>
       </c>
-      <c r="B10" s="216">
+      <c r="B10" s="213">
         <f>ROUND(SUM('工作表1'!F35:F36),6)</f>
         <v/>
       </c>
-      <c r="C10" s="216">
+      <c r="C10" s="213">
         <f>ROUND(SUM('工作表1'!K35:K36),6)</f>
         <v/>
       </c>
-      <c r="D10" s="216">
+      <c r="D10" s="213">
         <f>ROUND(SUM('工作表1'!P35:P36),6)</f>
         <v/>
       </c>
-      <c r="E10" s="216">
+      <c r="E10" s="213">
         <f>ROUND(SUM('工作表1'!U35:U36),6)</f>
         <v/>
       </c>
-      <c r="H10">
+      <c r="H10" s="0">
         <f>IF('工作表1'!D10="","",LEFT('工作表1'!D10,1))</f>
         <v/>
       </c>
-      <c r="I10">
+      <c r="I10" s="0">
         <f>IF(ISNUMBER('工作表1'!F10),'工作表1'!F10,0)</f>
         <v/>
       </c>
-      <c r="J10">
+      <c r="J10" s="0">
+        <f>IF('工作表1'!D10="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D10)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K10" s="0">
         <f>IF('工作表1'!I10="","",LEFT('工作表1'!I10,1))</f>
         <v/>
       </c>
-      <c r="K10">
+      <c r="L10" s="0">
         <f>IF(ISNUMBER('工作表1'!K10),'工作表1'!K10,0)</f>
         <v/>
       </c>
-      <c r="L10">
+      <c r="M10" s="0">
+        <f>IF('工作表1'!I10="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I10)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N10" s="0">
         <f>IF('工作表1'!N10="","",LEFT('工作表1'!N10,1))</f>
         <v/>
       </c>
-      <c r="M10">
+      <c r="O10" s="0">
         <f>IF(ISNUMBER('工作表1'!P10),'工作表1'!P10,0)</f>
         <v/>
       </c>
-      <c r="N10">
+      <c r="P10" s="0">
+        <f>IF('工作表1'!N10="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N10)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q10" s="0">
         <f>IF('工作表1'!S10="","",LEFT('工作表1'!S10,1))</f>
         <v/>
       </c>
-      <c r="O10">
+      <c r="R10" s="0">
         <f>IF(ISNUMBER('工作表1'!U10),'工作表1'!U10,0)</f>
+        <v/>
+      </c>
+      <c r="S10" s="0">
+        <f>IF('工作表1'!S10="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S10)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -6544,53 +6924,49 @@
           <t>5 ELIA（第38-39列）</t>
         </is>
       </c>
-      <c r="B11" s="216">
+      <c r="B11" s="213">
         <f>ROUND(SUM('工作表1'!F38:F39),6)</f>
         <v/>
       </c>
-      <c r="C11" s="216">
+      <c r="C11" s="213">
         <f>ROUND(SUM('工作表1'!K38:K39),6)</f>
         <v/>
       </c>
-      <c r="D11" s="216">
+      <c r="D11" s="213">
         <f>ROUND(SUM('工作表1'!P38:P39),6)</f>
         <v/>
       </c>
-      <c r="E11" s="216">
+      <c r="E11" s="213">
         <f>ROUND(SUM('工作表1'!U38:U39),6)</f>
         <v/>
       </c>
-      <c r="H11">
-        <f>IF('工作表1'!D11="","",LEFT('工作表1'!D11,1))</f>
-        <v/>
-      </c>
-      <c r="I11">
-        <f>IF(ISNUMBER('工作表1'!F11),'工作表1'!F11,0)</f>
-        <v/>
-      </c>
-      <c r="J11">
-        <f>IF('工作表1'!I11="","",LEFT('工作表1'!I11,1))</f>
-        <v/>
-      </c>
-      <c r="K11">
-        <f>IF(ISNUMBER('工作表1'!K11),'工作表1'!K11,0)</f>
-        <v/>
-      </c>
-      <c r="L11">
-        <f>IF('工作表1'!N11="","",LEFT('工作表1'!N11,1))</f>
-        <v/>
-      </c>
-      <c r="M11">
-        <f>IF(ISNUMBER('工作表1'!P11),'工作表1'!P11,0)</f>
-        <v/>
-      </c>
-      <c r="N11">
-        <f>IF('工作表1'!S11="","",LEFT('工作表1'!S11,1))</f>
-        <v/>
-      </c>
-      <c r="O11">
-        <f>IF(ISNUMBER('工作表1'!U11),'工作表1'!U11,0)</f>
-        <v/>
+      <c r="H11" s="0" t="inlineStr"/>
+      <c r="I11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="0" t="inlineStr"/>
+      <c r="L11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="0" t="inlineStr"/>
+      <c r="O11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="0" t="inlineStr"/>
+      <c r="R11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -6599,53 +6975,49 @@
           <t>6 支付AP（第42-43列）</t>
         </is>
       </c>
-      <c r="B12" s="216">
+      <c r="B12" s="213">
         <f>ROUND(SUM('工作表1'!F42:F43),6)</f>
         <v/>
       </c>
-      <c r="C12" s="216">
+      <c r="C12" s="213">
         <f>ROUND(SUM('工作表1'!K42:K43),6)</f>
         <v/>
       </c>
-      <c r="D12" s="216">
+      <c r="D12" s="213">
         <f>ROUND(SUM('工作表1'!P42:P43),6)</f>
         <v/>
       </c>
-      <c r="E12" s="216">
+      <c r="E12" s="213">
         <f>ROUND(SUM('工作表1'!U42:U43),6)</f>
         <v/>
       </c>
-      <c r="H12">
-        <f>IF('工作表1'!D12="","",LEFT('工作表1'!D12,1))</f>
-        <v/>
-      </c>
-      <c r="I12">
-        <f>IF(ISNUMBER('工作表1'!F12),'工作表1'!F12,0)</f>
-        <v/>
-      </c>
-      <c r="J12">
-        <f>IF('工作表1'!I12="","",LEFT('工作表1'!I12,1))</f>
-        <v/>
-      </c>
-      <c r="K12">
-        <f>IF(ISNUMBER('工作表1'!K12),'工作表1'!K12,0)</f>
-        <v/>
-      </c>
-      <c r="L12">
-        <f>IF('工作表1'!N12="","",LEFT('工作表1'!N12,1))</f>
-        <v/>
-      </c>
-      <c r="M12">
-        <f>IF(ISNUMBER('工作表1'!P12),'工作表1'!P12,0)</f>
-        <v/>
-      </c>
-      <c r="N12">
-        <f>IF('工作表1'!S12="","",LEFT('工作表1'!S12,1))</f>
-        <v/>
-      </c>
-      <c r="O12">
-        <f>IF(ISNUMBER('工作表1'!U12),'工作表1'!U12,0)</f>
-        <v/>
+      <c r="H12" s="0" t="inlineStr"/>
+      <c r="I12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="0" t="inlineStr"/>
+      <c r="L12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="0" t="inlineStr"/>
+      <c r="O12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="0" t="inlineStr"/>
+      <c r="R12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -6654,239 +7026,259 @@
           <t>7 收取AR（第45-46列）</t>
         </is>
       </c>
-      <c r="B13" s="216">
+      <c r="B13" s="213">
         <f>ROUND(SUM('工作表1'!F45:F46),6)</f>
         <v/>
       </c>
-      <c r="C13" s="216">
+      <c r="C13" s="213">
         <f>ROUND(SUM('工作表1'!K45:K46),6)</f>
         <v/>
       </c>
-      <c r="D13" s="216">
+      <c r="D13" s="213">
         <f>ROUND(SUM('工作表1'!P45:P46),6)</f>
         <v/>
       </c>
-      <c r="E13" s="216">
+      <c r="E13" s="213">
         <f>ROUND(SUM('工作表1'!U45:U46),6)</f>
         <v/>
       </c>
-      <c r="H13">
-        <f>IF('工作表1'!D13="","",LEFT('工作表1'!D13,1))</f>
-        <v/>
-      </c>
-      <c r="I13">
-        <f>IF(ISNUMBER('工作表1'!F13),'工作表1'!F13,0)</f>
-        <v/>
-      </c>
-      <c r="J13">
-        <f>IF('工作表1'!I13="","",LEFT('工作表1'!I13,1))</f>
-        <v/>
-      </c>
-      <c r="K13">
-        <f>IF(ISNUMBER('工作表1'!K13),'工作表1'!K13,0)</f>
-        <v/>
-      </c>
-      <c r="L13">
-        <f>IF('工作表1'!N13="","",LEFT('工作表1'!N13,1))</f>
-        <v/>
-      </c>
-      <c r="M13">
-        <f>IF(ISNUMBER('工作表1'!P13),'工作表1'!P13,0)</f>
-        <v/>
-      </c>
-      <c r="N13">
-        <f>IF('工作表1'!S13="","",LEFT('工作表1'!S13,1))</f>
-        <v/>
-      </c>
-      <c r="O13">
-        <f>IF(ISNUMBER('工作表1'!U13),'工作表1'!U13,0)</f>
-        <v/>
+      <c r="H13" s="0" t="inlineStr"/>
+      <c r="I13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="0" t="inlineStr"/>
+      <c r="L13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="0" t="inlineStr"/>
+      <c r="O13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="0" t="inlineStr"/>
+      <c r="R13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="215" t="inlineStr">
+      <c r="A14" s="212" t="inlineStr">
         <is>
           <t>A 結果</t>
         </is>
       </c>
-      <c r="B14" s="217">
+      <c r="B14" s="214">
         <f>IF(SUMPRODUCT(ABS(B3:B13))&lt;0.000001,"OK","不平")</f>
         <v/>
       </c>
-      <c r="C14" s="217">
+      <c r="C14" s="214">
         <f>IF(SUMPRODUCT(ABS(C3:C13))&lt;0.000001,"OK","不平")</f>
         <v/>
       </c>
-      <c r="D14" s="217">
+      <c r="D14" s="214">
         <f>IF(SUMPRODUCT(ABS(D3:D13))&lt;0.000001,"OK","不平")</f>
         <v/>
       </c>
-      <c r="E14" s="217">
+      <c r="E14" s="214">
         <f>IF(SUMPRODUCT(ABS(E3:E13))&lt;0.000001,"OK","不平")</f>
         <v/>
       </c>
-      <c r="H14">
-        <f>IF('工作表1'!D14="","",LEFT('工作表1'!D14,1))</f>
-        <v/>
-      </c>
-      <c r="I14">
-        <f>IF(ISNUMBER('工作表1'!F14),'工作表1'!F14,0)</f>
-        <v/>
-      </c>
-      <c r="J14">
-        <f>IF('工作表1'!I14="","",LEFT('工作表1'!I14,1))</f>
-        <v/>
-      </c>
-      <c r="K14">
-        <f>IF(ISNUMBER('工作表1'!K14),'工作表1'!K14,0)</f>
-        <v/>
-      </c>
-      <c r="L14">
-        <f>IF('工作表1'!N14="","",LEFT('工作表1'!N14,1))</f>
-        <v/>
-      </c>
-      <c r="M14">
-        <f>IF(ISNUMBER('工作表1'!P14),'工作表1'!P14,0)</f>
-        <v/>
-      </c>
-      <c r="N14">
-        <f>IF('工作表1'!S14="","",LEFT('工作表1'!S14,1))</f>
-        <v/>
-      </c>
-      <c r="O14">
-        <f>IF(ISNUMBER('工作表1'!U14),'工作表1'!U14,0)</f>
-        <v/>
+      <c r="H14" s="0" t="inlineStr"/>
+      <c r="I14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="0" t="inlineStr"/>
+      <c r="L14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="0" t="inlineStr"/>
+      <c r="O14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="0" t="inlineStr"/>
+      <c r="R14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="H15">
-        <f>IF('工作表1'!D15="","",LEFT('工作表1'!D15,1))</f>
-        <v/>
-      </c>
-      <c r="I15">
-        <f>IF(ISNUMBER('工作表1'!F15),'工作表1'!F15,0)</f>
-        <v/>
-      </c>
-      <c r="J15">
-        <f>IF('工作表1'!I15="","",LEFT('工作表1'!I15,1))</f>
-        <v/>
-      </c>
-      <c r="K15">
-        <f>IF(ISNUMBER('工作表1'!K15),'工作表1'!K15,0)</f>
-        <v/>
-      </c>
-      <c r="L15">
-        <f>IF('工作表1'!N15="","",LEFT('工作表1'!N15,1))</f>
-        <v/>
-      </c>
-      <c r="M15">
-        <f>IF(ISNUMBER('工作表1'!P15),'工作表1'!P15,0)</f>
-        <v/>
-      </c>
-      <c r="N15">
-        <f>IF('工作表1'!S15="","",LEFT('工作表1'!S15,1))</f>
-        <v/>
-      </c>
-      <c r="O15">
-        <f>IF(ISNUMBER('工作表1'!U15),'工作表1'!U15,0)</f>
-        <v/>
+      <c r="H15" s="0" t="inlineStr"/>
+      <c r="I15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="0" t="inlineStr"/>
+      <c r="L15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="0" t="inlineStr"/>
+      <c r="O15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="0" t="inlineStr"/>
+      <c r="R15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="215" t="inlineStr">
-        <is>
-          <t>B. 期末總結 vs 分錄直接加總（依科目代號首碼：1/2=B/S，4/5/6=P/L）</t>
-        </is>
-      </c>
-      <c r="H16">
+      <c r="A16" s="212" t="inlineStr">
+        <is>
+          <t>B. 期末總結 vs BIM分錄直接加總（只計BIM列；代號首碼1/2=B/S，4/5/6=P/L）</t>
+        </is>
+      </c>
+      <c r="H16" s="0">
         <f>IF('工作表1'!D16="","",LEFT('工作表1'!D16,1))</f>
         <v/>
       </c>
-      <c r="I16">
+      <c r="I16" s="0">
         <f>IF(ISNUMBER('工作表1'!F16),'工作表1'!F16,0)</f>
         <v/>
       </c>
-      <c r="J16">
+      <c r="J16" s="0">
+        <f>IF('工作表1'!D16="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D16)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K16" s="0">
         <f>IF('工作表1'!I16="","",LEFT('工作表1'!I16,1))</f>
         <v/>
       </c>
-      <c r="K16">
+      <c r="L16" s="0">
         <f>IF(ISNUMBER('工作表1'!K16),'工作表1'!K16,0)</f>
         <v/>
       </c>
-      <c r="L16">
+      <c r="M16" s="0">
+        <f>IF('工作表1'!I16="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I16)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N16" s="0">
         <f>IF('工作表1'!N16="","",LEFT('工作表1'!N16,1))</f>
         <v/>
       </c>
-      <c r="M16">
+      <c r="O16" s="0">
         <f>IF(ISNUMBER('工作表1'!P16),'工作表1'!P16,0)</f>
         <v/>
       </c>
-      <c r="N16">
+      <c r="P16" s="0">
+        <f>IF('工作表1'!N16="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N16)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q16" s="0">
         <f>IF('工作表1'!S16="","",LEFT('工作表1'!S16,1))</f>
         <v/>
       </c>
-      <c r="O16">
+      <c r="R16" s="0">
         <f>IF(ISNUMBER('工作表1'!U16),'工作表1'!U16,0)</f>
         <v/>
       </c>
+      <c r="S16" s="0">
+        <f>IF('工作表1'!S16="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S16)&gt;0,0,1))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="215" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B17" s="215" t="inlineStr">
+      <c r="B17" s="212" t="inlineStr">
         <is>
           <t>內案POC</t>
         </is>
       </c>
-      <c r="C17" s="215" t="inlineStr">
+      <c r="C17" s="212" t="inlineStr">
         <is>
           <t>外案POC</t>
         </is>
       </c>
-      <c r="D17" s="215" t="inlineStr">
+      <c r="D17" s="212" t="inlineStr">
         <is>
           <t>雜項</t>
         </is>
       </c>
-      <c r="E17" s="215" t="inlineStr">
+      <c r="E17" s="212" t="inlineStr">
         <is>
           <t>備標</t>
         </is>
       </c>
-      <c r="H17">
+      <c r="H17" s="0">
         <f>IF('工作表1'!D17="","",LEFT('工作表1'!D17,1))</f>
         <v/>
       </c>
-      <c r="I17">
+      <c r="I17" s="0">
         <f>IF(ISNUMBER('工作表1'!F17),'工作表1'!F17,0)</f>
         <v/>
       </c>
-      <c r="J17">
+      <c r="J17" s="0">
+        <f>IF('工作表1'!D17="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D17)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K17" s="0">
         <f>IF('工作表1'!I17="","",LEFT('工作表1'!I17,1))</f>
         <v/>
       </c>
-      <c r="K17">
+      <c r="L17" s="0">
         <f>IF(ISNUMBER('工作表1'!K17),'工作表1'!K17,0)</f>
         <v/>
       </c>
-      <c r="L17">
+      <c r="M17" s="0">
+        <f>IF('工作表1'!I17="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I17)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N17" s="0">
         <f>IF('工作表1'!N17="","",LEFT('工作表1'!N17,1))</f>
         <v/>
       </c>
-      <c r="M17">
+      <c r="O17" s="0">
         <f>IF(ISNUMBER('工作表1'!P17),'工作表1'!P17,0)</f>
         <v/>
       </c>
-      <c r="N17">
+      <c r="P17" s="0">
+        <f>IF('工作表1'!N17="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N17)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q17" s="0">
         <f>IF('工作表1'!S17="","",LEFT('工作表1'!S17,1))</f>
         <v/>
       </c>
-      <c r="O17">
+      <c r="R17" s="0">
         <f>IF(ISNUMBER('工作表1'!U17),'工作表1'!U17,0)</f>
+        <v/>
+      </c>
+      <c r="S17" s="0">
+        <f>IF('工作表1'!S17="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S17)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -6896,107 +7288,139 @@
           <t>B/S 分錄加總</t>
         </is>
       </c>
-      <c r="B18" s="218">
+      <c r="B18" s="215">
         <f>SUMIF($H$4:$H$47,"1",$I$4:$I$47)+SUMIF($H$4:$H$47,"2",$I$4:$I$47)</f>
         <v/>
       </c>
-      <c r="C18" s="218">
-        <f>SUMIF($J$4:$J$47,"1",$K$4:$K$47)+SUMIF($J$4:$J$47,"2",$K$4:$K$47)</f>
-        <v/>
-      </c>
-      <c r="D18" s="218">
-        <f>SUMIF($L$4:$L$47,"1",$M$4:$M$47)+SUMIF($L$4:$L$47,"2",$M$4:$M$47)</f>
-        <v/>
-      </c>
-      <c r="E18" s="218">
+      <c r="C18" s="215">
+        <f>SUMIF($K$4:$K$47,"1",$L$4:$L$47)+SUMIF($K$4:$K$47,"2",$L$4:$L$47)</f>
+        <v/>
+      </c>
+      <c r="D18" s="215">
         <f>SUMIF($N$4:$N$47,"1",$O$4:$O$47)+SUMIF($N$4:$N$47,"2",$O$4:$O$47)</f>
         <v/>
       </c>
-      <c r="H18">
+      <c r="E18" s="215">
+        <f>SUMIF($Q$4:$Q$47,"1",$R$4:$R$47)+SUMIF($Q$4:$Q$47,"2",$R$4:$R$47)</f>
+        <v/>
+      </c>
+      <c r="H18" s="0">
         <f>IF('工作表1'!D18="","",LEFT('工作表1'!D18,1))</f>
         <v/>
       </c>
-      <c r="I18">
+      <c r="I18" s="0">
         <f>IF(ISNUMBER('工作表1'!F18),'工作表1'!F18,0)</f>
         <v/>
       </c>
-      <c r="J18">
+      <c r="J18" s="0">
+        <f>IF('工作表1'!D18="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D18)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K18" s="0">
         <f>IF('工作表1'!I18="","",LEFT('工作表1'!I18,1))</f>
         <v/>
       </c>
-      <c r="K18">
+      <c r="L18" s="0">
         <f>IF(ISNUMBER('工作表1'!K18),'工作表1'!K18,0)</f>
         <v/>
       </c>
-      <c r="L18">
+      <c r="M18" s="0">
+        <f>IF('工作表1'!I18="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I18)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N18" s="0">
         <f>IF('工作表1'!N18="","",LEFT('工作表1'!N18,1))</f>
         <v/>
       </c>
-      <c r="M18">
+      <c r="O18" s="0">
         <f>IF(ISNUMBER('工作表1'!P18),'工作表1'!P18,0)</f>
         <v/>
       </c>
-      <c r="N18">
+      <c r="P18" s="0">
+        <f>IF('工作表1'!N18="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N18)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q18" s="0">
         <f>IF('工作表1'!S18="","",LEFT('工作表1'!S18,1))</f>
         <v/>
       </c>
-      <c r="O18">
+      <c r="R18" s="0">
         <f>IF(ISNUMBER('工作表1'!U18),'工作表1'!U18,0)</f>
+        <v/>
+      </c>
+      <c r="S18" s="0">
+        <f>IF('工作表1'!S18="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S18)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>B/S 期末總結(F50+F53:F57)</t>
-        </is>
-      </c>
-      <c r="B19" s="218">
+          <t>B/S 期末總結(總計欄50+53:57)</t>
+        </is>
+      </c>
+      <c r="B19" s="215">
         <f>'工作表1'!F50+SUM('工作表1'!F53:F57)</f>
         <v/>
       </c>
-      <c r="C19" s="218">
+      <c r="C19" s="215">
         <f>'工作表1'!K50+SUM('工作表1'!K53:K57)</f>
         <v/>
       </c>
-      <c r="D19" s="218">
+      <c r="D19" s="215">
         <f>'工作表1'!P50+SUM('工作表1'!P53:P57)</f>
         <v/>
       </c>
-      <c r="E19" s="218">
+      <c r="E19" s="215">
         <f>'工作表1'!U50+SUM('工作表1'!U53:U57)</f>
         <v/>
       </c>
-      <c r="H19">
+      <c r="H19" s="0">
         <f>IF('工作表1'!D19="","",LEFT('工作表1'!D19,1))</f>
         <v/>
       </c>
-      <c r="I19">
+      <c r="I19" s="0">
         <f>IF(ISNUMBER('工作表1'!F19),'工作表1'!F19,0)</f>
         <v/>
       </c>
-      <c r="J19">
+      <c r="J19" s="0">
+        <f>IF('工作表1'!D19="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D19)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K19" s="0">
         <f>IF('工作表1'!I19="","",LEFT('工作表1'!I19,1))</f>
         <v/>
       </c>
-      <c r="K19">
+      <c r="L19" s="0">
         <f>IF(ISNUMBER('工作表1'!K19),'工作表1'!K19,0)</f>
         <v/>
       </c>
-      <c r="L19">
+      <c r="M19" s="0">
+        <f>IF('工作表1'!I19="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I19)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N19" s="0">
         <f>IF('工作表1'!N19="","",LEFT('工作表1'!N19,1))</f>
         <v/>
       </c>
-      <c r="M19">
+      <c r="O19" s="0">
         <f>IF(ISNUMBER('工作表1'!P19),'工作表1'!P19,0)</f>
         <v/>
       </c>
-      <c r="N19">
+      <c r="P19" s="0">
+        <f>IF('工作表1'!N19="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N19)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q19" s="0">
         <f>IF('工作表1'!S19="","",LEFT('工作表1'!S19,1))</f>
         <v/>
       </c>
-      <c r="O19">
+      <c r="R19" s="0">
         <f>IF(ISNUMBER('工作表1'!U19),'工作表1'!U19,0)</f>
+        <v/>
+      </c>
+      <c r="S19" s="0">
+        <f>IF('工作表1'!S19="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S19)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -7006,107 +7430,139 @@
           <t>P/L 分錄加總</t>
         </is>
       </c>
-      <c r="B20" s="218">
+      <c r="B20" s="215">
         <f>SUMIF($H$4:$H$47,"4",$I$4:$I$47)+SUMIF($H$4:$H$47,"5",$I$4:$I$47)+SUMIF($H$4:$H$47,"6",$I$4:$I$47)</f>
         <v/>
       </c>
-      <c r="C20" s="218">
-        <f>SUMIF($J$4:$J$47,"4",$K$4:$K$47)+SUMIF($J$4:$J$47,"5",$K$4:$K$47)+SUMIF($J$4:$J$47,"6",$K$4:$K$47)</f>
-        <v/>
-      </c>
-      <c r="D20" s="218">
-        <f>SUMIF($L$4:$L$47,"4",$M$4:$M$47)+SUMIF($L$4:$L$47,"5",$M$4:$M$47)+SUMIF($L$4:$L$47,"6",$M$4:$M$47)</f>
-        <v/>
-      </c>
-      <c r="E20" s="218">
+      <c r="C20" s="215">
+        <f>SUMIF($K$4:$K$47,"4",$L$4:$L$47)+SUMIF($K$4:$K$47,"5",$L$4:$L$47)+SUMIF($K$4:$K$47,"6",$L$4:$L$47)</f>
+        <v/>
+      </c>
+      <c r="D20" s="215">
         <f>SUMIF($N$4:$N$47,"4",$O$4:$O$47)+SUMIF($N$4:$N$47,"5",$O$4:$O$47)+SUMIF($N$4:$N$47,"6",$O$4:$O$47)</f>
         <v/>
       </c>
-      <c r="H20">
+      <c r="E20" s="215">
+        <f>SUMIF($Q$4:$Q$47,"4",$R$4:$R$47)+SUMIF($Q$4:$Q$47,"5",$R$4:$R$47)+SUMIF($Q$4:$Q$47,"6",$R$4:$R$47)</f>
+        <v/>
+      </c>
+      <c r="H20" s="0">
         <f>IF('工作表1'!D20="","",LEFT('工作表1'!D20,1))</f>
         <v/>
       </c>
-      <c r="I20">
+      <c r="I20" s="0">
         <f>IF(ISNUMBER('工作表1'!F20),'工作表1'!F20,0)</f>
         <v/>
       </c>
-      <c r="J20">
+      <c r="J20" s="0">
+        <f>IF('工作表1'!D20="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D20)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K20" s="0">
         <f>IF('工作表1'!I20="","",LEFT('工作表1'!I20,1))</f>
         <v/>
       </c>
-      <c r="K20">
+      <c r="L20" s="0">
         <f>IF(ISNUMBER('工作表1'!K20),'工作表1'!K20,0)</f>
         <v/>
       </c>
-      <c r="L20">
+      <c r="M20" s="0">
+        <f>IF('工作表1'!I20="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I20)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N20" s="0">
         <f>IF('工作表1'!N20="","",LEFT('工作表1'!N20,1))</f>
         <v/>
       </c>
-      <c r="M20">
+      <c r="O20" s="0">
         <f>IF(ISNUMBER('工作表1'!P20),'工作表1'!P20,0)</f>
         <v/>
       </c>
-      <c r="N20">
+      <c r="P20" s="0">
+        <f>IF('工作表1'!N20="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N20)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q20" s="0">
         <f>IF('工作表1'!S20="","",LEFT('工作表1'!S20,1))</f>
         <v/>
       </c>
-      <c r="O20">
+      <c r="R20" s="0">
         <f>IF(ISNUMBER('工作表1'!U20),'工作表1'!U20,0)</f>
+        <v/>
+      </c>
+      <c r="S20" s="0">
+        <f>IF('工作表1'!S20="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S20)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>P/L 期末總結(F58)</t>
-        </is>
-      </c>
-      <c r="B21" s="218">
+          <t>P/L 期末總結(總計欄58)</t>
+        </is>
+      </c>
+      <c r="B21" s="215">
         <f>'工作表1'!F58</f>
         <v/>
       </c>
-      <c r="C21" s="218">
+      <c r="C21" s="215">
         <f>'工作表1'!K58</f>
         <v/>
       </c>
-      <c r="D21" s="218">
+      <c r="D21" s="215">
         <f>'工作表1'!P58</f>
         <v/>
       </c>
-      <c r="E21" s="218">
+      <c r="E21" s="215">
         <f>'工作表1'!U58</f>
         <v/>
       </c>
-      <c r="H21">
+      <c r="H21" s="0">
         <f>IF('工作表1'!D21="","",LEFT('工作表1'!D21,1))</f>
         <v/>
       </c>
-      <c r="I21">
+      <c r="I21" s="0">
         <f>IF(ISNUMBER('工作表1'!F21),'工作表1'!F21,0)</f>
         <v/>
       </c>
-      <c r="J21">
+      <c r="J21" s="0">
+        <f>IF('工作表1'!D21="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D21)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K21" s="0">
         <f>IF('工作表1'!I21="","",LEFT('工作表1'!I21,1))</f>
         <v/>
       </c>
-      <c r="K21">
+      <c r="L21" s="0">
         <f>IF(ISNUMBER('工作表1'!K21),'工作表1'!K21,0)</f>
         <v/>
       </c>
-      <c r="L21">
+      <c r="M21" s="0">
+        <f>IF('工作表1'!I21="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I21)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N21" s="0">
         <f>IF('工作表1'!N21="","",LEFT('工作表1'!N21,1))</f>
         <v/>
       </c>
-      <c r="M21">
+      <c r="O21" s="0">
         <f>IF(ISNUMBER('工作表1'!P21),'工作表1'!P21,0)</f>
         <v/>
       </c>
-      <c r="N21">
+      <c r="P21" s="0">
+        <f>IF('工作表1'!N21="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N21)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q21" s="0">
         <f>IF('工作表1'!S21="","",LEFT('工作表1'!S21,1))</f>
         <v/>
       </c>
-      <c r="O21">
+      <c r="R21" s="0">
         <f>IF(ISNUMBER('工作表1'!U21),'工作表1'!U21,0)</f>
+        <v/>
+      </c>
+      <c r="S21" s="0">
+        <f>IF('工作表1'!S21="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S21)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -7116,52 +7572,68 @@
           <t>B/S 差異</t>
         </is>
       </c>
-      <c r="B22" s="218">
+      <c r="B22" s="215">
         <f>B19-B18</f>
         <v/>
       </c>
-      <c r="C22" s="218">
+      <c r="C22" s="215">
         <f>C19-C18</f>
         <v/>
       </c>
-      <c r="D22" s="218">
+      <c r="D22" s="215">
         <f>D19-D18</f>
         <v/>
       </c>
-      <c r="E22" s="218">
+      <c r="E22" s="215">
         <f>E19-E18</f>
         <v/>
       </c>
-      <c r="H22">
+      <c r="H22" s="0">
         <f>IF('工作表1'!D22="","",LEFT('工作表1'!D22,1))</f>
         <v/>
       </c>
-      <c r="I22">
+      <c r="I22" s="0">
         <f>IF(ISNUMBER('工作表1'!F22),'工作表1'!F22,0)</f>
         <v/>
       </c>
-      <c r="J22">
+      <c r="J22" s="0">
+        <f>IF('工作表1'!D22="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D22)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K22" s="0">
         <f>IF('工作表1'!I22="","",LEFT('工作表1'!I22,1))</f>
         <v/>
       </c>
-      <c r="K22">
+      <c r="L22" s="0">
         <f>IF(ISNUMBER('工作表1'!K22),'工作表1'!K22,0)</f>
         <v/>
       </c>
-      <c r="L22">
+      <c r="M22" s="0">
+        <f>IF('工作表1'!I22="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I22)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N22" s="0">
         <f>IF('工作表1'!N22="","",LEFT('工作表1'!N22,1))</f>
         <v/>
       </c>
-      <c r="M22">
+      <c r="O22" s="0">
         <f>IF(ISNUMBER('工作表1'!P22),'工作表1'!P22,0)</f>
         <v/>
       </c>
-      <c r="N22">
+      <c r="P22" s="0">
+        <f>IF('工作表1'!N22="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N22)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q22" s="0">
         <f>IF('工作表1'!S22="","",LEFT('工作表1'!S22,1))</f>
         <v/>
       </c>
-      <c r="O22">
+      <c r="R22" s="0">
         <f>IF(ISNUMBER('工作表1'!U22),'工作表1'!U22,0)</f>
+        <v/>
+      </c>
+      <c r="S22" s="0">
+        <f>IF('工作表1'!S22="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S22)&gt;0,0,1))</f>
         <v/>
       </c>
     </row>
@@ -7171,53 +7643,49 @@
           <t>P/L 差異</t>
         </is>
       </c>
-      <c r="B23" s="218">
+      <c r="B23" s="215">
         <f>B21-B20</f>
         <v/>
       </c>
-      <c r="C23" s="218">
+      <c r="C23" s="215">
         <f>C21-C20</f>
         <v/>
       </c>
-      <c r="D23" s="218">
+      <c r="D23" s="215">
         <f>D21-D20</f>
         <v/>
       </c>
-      <c r="E23" s="218">
+      <c r="E23" s="215">
         <f>E21-E20</f>
         <v/>
       </c>
-      <c r="H23">
-        <f>IF('工作表1'!D23="","",LEFT('工作表1'!D23,1))</f>
-        <v/>
-      </c>
-      <c r="I23">
-        <f>IF(ISNUMBER('工作表1'!F23),'工作表1'!F23,0)</f>
-        <v/>
-      </c>
-      <c r="J23">
-        <f>IF('工作表1'!I23="","",LEFT('工作表1'!I23,1))</f>
-        <v/>
-      </c>
-      <c r="K23">
-        <f>IF(ISNUMBER('工作表1'!K23),'工作表1'!K23,0)</f>
-        <v/>
-      </c>
-      <c r="L23">
-        <f>IF('工作表1'!N23="","",LEFT('工作表1'!N23,1))</f>
-        <v/>
-      </c>
-      <c r="M23">
-        <f>IF(ISNUMBER('工作表1'!P23),'工作表1'!P23,0)</f>
-        <v/>
-      </c>
-      <c r="N23">
-        <f>IF('工作表1'!S23="","",LEFT('工作表1'!S23,1))</f>
-        <v/>
-      </c>
-      <c r="O23">
-        <f>IF(ISNUMBER('工作表1'!U23),'工作表1'!U23,0)</f>
-        <v/>
+      <c r="H23" s="0" t="inlineStr"/>
+      <c r="I23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="0" t="inlineStr"/>
+      <c r="L23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="0" t="inlineStr"/>
+      <c r="O23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="0" t="inlineStr"/>
+      <c r="R23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -7226,53 +7694,49 @@
           <t>B/S+P/L(應為0)</t>
         </is>
       </c>
-      <c r="B24" s="218">
+      <c r="B24" s="215">
         <f>B19+B21</f>
         <v/>
       </c>
-      <c r="C24" s="218">
+      <c r="C24" s="215">
         <f>C19+C21</f>
         <v/>
       </c>
-      <c r="D24" s="218">
+      <c r="D24" s="215">
         <f>D19+D21</f>
         <v/>
       </c>
-      <c r="E24" s="218">
+      <c r="E24" s="215">
         <f>E19+E21</f>
         <v/>
       </c>
-      <c r="H24">
-        <f>IF('工作表1'!D24="","",LEFT('工作表1'!D24,1))</f>
-        <v/>
-      </c>
-      <c r="I24">
-        <f>IF(ISNUMBER('工作表1'!F24),'工作表1'!F24,0)</f>
-        <v/>
-      </c>
-      <c r="J24">
-        <f>IF('工作表1'!I24="","",LEFT('工作表1'!I24,1))</f>
-        <v/>
-      </c>
-      <c r="K24">
-        <f>IF(ISNUMBER('工作表1'!K24),'工作表1'!K24,0)</f>
-        <v/>
-      </c>
-      <c r="L24">
-        <f>IF('工作表1'!N24="","",LEFT('工作表1'!N24,1))</f>
-        <v/>
-      </c>
-      <c r="M24">
-        <f>IF(ISNUMBER('工作表1'!P24),'工作表1'!P24,0)</f>
-        <v/>
-      </c>
-      <c r="N24">
-        <f>IF('工作表1'!S24="","",LEFT('工作表1'!S24,1))</f>
-        <v/>
-      </c>
-      <c r="O24">
-        <f>IF(ISNUMBER('工作表1'!U24),'工作表1'!U24,0)</f>
-        <v/>
+      <c r="H24" s="0" t="inlineStr"/>
+      <c r="I24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="0" t="inlineStr"/>
+      <c r="L24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="0" t="inlineStr"/>
+      <c r="O24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="0" t="inlineStr"/>
+      <c r="R24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -7281,801 +7745,911 @@
           <t>B 結果</t>
         </is>
       </c>
-      <c r="B25" s="219">
+      <c r="B25" s="214">
         <f>IF(AND(ABS(B22)&lt;0.000001,ABS(B23)&lt;0.000001,ABS(B24)&lt;0.000001),"OK","不符")</f>
         <v/>
       </c>
-      <c r="C25" s="219">
+      <c r="C25" s="214">
         <f>IF(AND(ABS(C22)&lt;0.000001,ABS(C23)&lt;0.000001,ABS(C24)&lt;0.000001),"OK","不符")</f>
         <v/>
       </c>
-      <c r="D25" s="219">
+      <c r="D25" s="214">
         <f>IF(AND(ABS(D22)&lt;0.000001,ABS(D23)&lt;0.000001,ABS(D24)&lt;0.000001),"OK","不符")</f>
         <v/>
       </c>
-      <c r="E25" s="219">
+      <c r="E25" s="214">
         <f>IF(AND(ABS(E22)&lt;0.000001,ABS(E23)&lt;0.000001,ABS(E24)&lt;0.000001),"OK","不符")</f>
         <v/>
       </c>
-      <c r="H25">
-        <f>IF('工作表1'!D25="","",LEFT('工作表1'!D25,1))</f>
-        <v/>
-      </c>
-      <c r="I25">
-        <f>IF(ISNUMBER('工作表1'!F25),'工作表1'!F25,0)</f>
-        <v/>
-      </c>
-      <c r="J25">
-        <f>IF('工作表1'!I25="","",LEFT('工作表1'!I25,1))</f>
-        <v/>
-      </c>
-      <c r="K25">
-        <f>IF(ISNUMBER('工作表1'!K25),'工作表1'!K25,0)</f>
-        <v/>
-      </c>
-      <c r="L25">
-        <f>IF('工作表1'!N25="","",LEFT('工作表1'!N25,1))</f>
-        <v/>
-      </c>
-      <c r="M25">
-        <f>IF(ISNUMBER('工作表1'!P25),'工作表1'!P25,0)</f>
-        <v/>
-      </c>
-      <c r="N25">
-        <f>IF('工作表1'!S25="","",LEFT('工作表1'!S25,1))</f>
-        <v/>
-      </c>
-      <c r="O25">
-        <f>IF(ISNUMBER('工作表1'!U25),'工作表1'!U25,0)</f>
-        <v/>
+      <c r="H25" s="0" t="inlineStr"/>
+      <c r="I25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="0" t="inlineStr"/>
+      <c r="L25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="0" t="inlineStr"/>
+      <c r="O25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="0" t="inlineStr"/>
+      <c r="R25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
-      <c r="H26">
-        <f>IF('工作表1'!D26="","",LEFT('工作表1'!D26,1))</f>
-        <v/>
-      </c>
-      <c r="I26">
-        <f>IF(ISNUMBER('工作表1'!F26),'工作表1'!F26,0)</f>
-        <v/>
-      </c>
-      <c r="J26">
-        <f>IF('工作表1'!I26="","",LEFT('工作表1'!I26,1))</f>
-        <v/>
-      </c>
-      <c r="K26">
-        <f>IF(ISNUMBER('工作表1'!K26),'工作表1'!K26,0)</f>
-        <v/>
-      </c>
-      <c r="L26">
-        <f>IF('工作表1'!N26="","",LEFT('工作表1'!N26,1))</f>
-        <v/>
-      </c>
-      <c r="M26">
-        <f>IF(ISNUMBER('工作表1'!P26),'工作表1'!P26,0)</f>
-        <v/>
-      </c>
-      <c r="N26">
-        <f>IF('工作表1'!S26="","",LEFT('工作表1'!S26,1))</f>
-        <v/>
-      </c>
-      <c r="O26">
-        <f>IF(ISNUMBER('工作表1'!U26),'工作表1'!U26,0)</f>
-        <v/>
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>C. BIM分錄科目未列入期末總結的行數</t>
+        </is>
+      </c>
+      <c r="B26" s="0">
+        <f>SUM($J$4:$J$47)</f>
+        <v/>
+      </c>
+      <c r="C26" s="0">
+        <f>SUM($M$4:$M$47)</f>
+        <v/>
+      </c>
+      <c r="D26" s="0">
+        <f>SUM($P$4:$P$47)</f>
+        <v/>
+      </c>
+      <c r="E26" s="0">
+        <f>SUM($S$4:$S$47)</f>
+        <v/>
+      </c>
+      <c r="H26" s="0" t="inlineStr"/>
+      <c r="I26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="0" t="inlineStr"/>
+      <c r="L26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="0" t="inlineStr"/>
+      <c r="O26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="0" t="inlineStr"/>
+      <c r="R26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
-      <c r="H27">
-        <f>IF('工作表1'!D27="","",LEFT('工作表1'!D27,1))</f>
-        <v/>
-      </c>
-      <c r="I27">
-        <f>IF(ISNUMBER('工作表1'!F27),'工作表1'!F27,0)</f>
-        <v/>
-      </c>
-      <c r="J27">
-        <f>IF('工作表1'!I27="","",LEFT('工作表1'!I27,1))</f>
-        <v/>
-      </c>
-      <c r="K27">
-        <f>IF(ISNUMBER('工作表1'!K27),'工作表1'!K27,0)</f>
-        <v/>
-      </c>
-      <c r="L27">
-        <f>IF('工作表1'!N27="","",LEFT('工作表1'!N27,1))</f>
-        <v/>
-      </c>
-      <c r="M27">
-        <f>IF(ISNUMBER('工作表1'!P27),'工作表1'!P27,0)</f>
-        <v/>
-      </c>
-      <c r="N27">
-        <f>IF('工作表1'!S27="","",LEFT('工作表1'!S27,1))</f>
-        <v/>
-      </c>
-      <c r="O27">
-        <f>IF(ISNUMBER('工作表1'!U27),'工作表1'!U27,0)</f>
-        <v/>
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>C 結果</t>
+        </is>
+      </c>
+      <c r="B27" s="214">
+        <f>IF(B26=0,"OK","有漏列")</f>
+        <v/>
+      </c>
+      <c r="C27" s="214">
+        <f>IF(C26=0,"OK","有漏列")</f>
+        <v/>
+      </c>
+      <c r="D27" s="214">
+        <f>IF(D26=0,"OK","有漏列")</f>
+        <v/>
+      </c>
+      <c r="E27" s="214">
+        <f>IF(E26=0,"OK","有漏列")</f>
+        <v/>
+      </c>
+      <c r="H27" s="0" t="inlineStr"/>
+      <c r="I27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="0" t="inlineStr"/>
+      <c r="L27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="0" t="inlineStr"/>
+      <c r="O27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="0" t="inlineStr"/>
+      <c r="R27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
-      <c r="H28">
-        <f>IF('工作表1'!D28="","",LEFT('工作表1'!D28,1))</f>
-        <v/>
-      </c>
-      <c r="I28">
-        <f>IF(ISNUMBER('工作表1'!F28),'工作表1'!F28,0)</f>
-        <v/>
-      </c>
-      <c r="J28">
-        <f>IF('工作表1'!I28="","",LEFT('工作表1'!I28,1))</f>
-        <v/>
-      </c>
-      <c r="K28">
-        <f>IF(ISNUMBER('工作表1'!K28),'工作表1'!K28,0)</f>
-        <v/>
-      </c>
-      <c r="L28">
-        <f>IF('工作表1'!N28="","",LEFT('工作表1'!N28,1))</f>
-        <v/>
-      </c>
-      <c r="M28">
-        <f>IF(ISNUMBER('工作表1'!P28),'工作表1'!P28,0)</f>
-        <v/>
-      </c>
-      <c r="N28">
-        <f>IF('工作表1'!S28="","",LEFT('工作表1'!S28,1))</f>
-        <v/>
-      </c>
-      <c r="O28">
-        <f>IF(ISNUMBER('工作表1'!U28),'工作表1'!U28,0)</f>
-        <v/>
+      <c r="H28" s="0" t="inlineStr"/>
+      <c r="I28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="0" t="inlineStr"/>
+      <c r="L28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="0" t="inlineStr"/>
+      <c r="O28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="0" t="inlineStr"/>
+      <c r="R28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
-      <c r="H29">
-        <f>IF('工作表1'!D29="","",LEFT('工作表1'!D29,1))</f>
-        <v/>
-      </c>
-      <c r="I29">
-        <f>IF(ISNUMBER('工作表1'!F29),'工作表1'!F29,0)</f>
-        <v/>
-      </c>
-      <c r="J29">
-        <f>IF('工作表1'!I29="","",LEFT('工作表1'!I29,1))</f>
-        <v/>
-      </c>
-      <c r="K29">
-        <f>IF(ISNUMBER('工作表1'!K29),'工作表1'!K29,0)</f>
-        <v/>
-      </c>
-      <c r="L29">
-        <f>IF('工作表1'!N29="","",LEFT('工作表1'!N29,1))</f>
-        <v/>
-      </c>
-      <c r="M29">
-        <f>IF(ISNUMBER('工作表1'!P29),'工作表1'!P29,0)</f>
-        <v/>
-      </c>
-      <c r="N29">
-        <f>IF('工作表1'!S29="","",LEFT('工作表1'!S29,1))</f>
-        <v/>
-      </c>
-      <c r="O29">
-        <f>IF(ISNUMBER('工作表1'!U29),'工作表1'!U29,0)</f>
-        <v/>
+      <c r="H29" s="0" t="inlineStr"/>
+      <c r="I29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="0" t="inlineStr"/>
+      <c r="L29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="0" t="inlineStr"/>
+      <c r="O29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="0" t="inlineStr"/>
+      <c r="R29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
-      <c r="H30">
-        <f>IF('工作表1'!D30="","",LEFT('工作表1'!D30,1))</f>
-        <v/>
-      </c>
-      <c r="I30">
-        <f>IF(ISNUMBER('工作表1'!F30),'工作表1'!F30,0)</f>
-        <v/>
-      </c>
-      <c r="J30">
-        <f>IF('工作表1'!I30="","",LEFT('工作表1'!I30,1))</f>
-        <v/>
-      </c>
-      <c r="K30">
-        <f>IF(ISNUMBER('工作表1'!K30),'工作表1'!K30,0)</f>
-        <v/>
-      </c>
-      <c r="L30">
-        <f>IF('工作表1'!N30="","",LEFT('工作表1'!N30,1))</f>
-        <v/>
-      </c>
-      <c r="M30">
-        <f>IF(ISNUMBER('工作表1'!P30),'工作表1'!P30,0)</f>
-        <v/>
-      </c>
-      <c r="N30">
-        <f>IF('工作表1'!S30="","",LEFT('工作表1'!S30,1))</f>
-        <v/>
-      </c>
-      <c r="O30">
-        <f>IF(ISNUMBER('工作表1'!U30),'工作表1'!U30,0)</f>
-        <v/>
+      <c r="H30" s="0" t="inlineStr"/>
+      <c r="I30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="0" t="inlineStr"/>
+      <c r="L30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="0" t="inlineStr"/>
+      <c r="O30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="0" t="inlineStr"/>
+      <c r="R30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
-      <c r="H31">
+      <c r="H31" s="0">
         <f>IF('工作表1'!D31="","",LEFT('工作表1'!D31,1))</f>
         <v/>
       </c>
-      <c r="I31">
+      <c r="I31" s="0">
         <f>IF(ISNUMBER('工作表1'!F31),'工作表1'!F31,0)</f>
         <v/>
       </c>
-      <c r="J31">
+      <c r="J31" s="0">
+        <f>IF('工作表1'!D31="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D31)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K31" s="0">
         <f>IF('工作表1'!I31="","",LEFT('工作表1'!I31,1))</f>
         <v/>
       </c>
-      <c r="K31">
+      <c r="L31" s="0">
         <f>IF(ISNUMBER('工作表1'!K31),'工作表1'!K31,0)</f>
         <v/>
       </c>
-      <c r="L31">
+      <c r="M31" s="0">
+        <f>IF('工作表1'!I31="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I31)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N31" s="0">
         <f>IF('工作表1'!N31="","",LEFT('工作表1'!N31,1))</f>
         <v/>
       </c>
-      <c r="M31">
+      <c r="O31" s="0">
         <f>IF(ISNUMBER('工作表1'!P31),'工作表1'!P31,0)</f>
         <v/>
       </c>
-      <c r="N31">
+      <c r="P31" s="0">
+        <f>IF('工作表1'!N31="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N31)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q31" s="0">
         <f>IF('工作表1'!S31="","",LEFT('工作表1'!S31,1))</f>
         <v/>
       </c>
-      <c r="O31">
+      <c r="R31" s="0">
         <f>IF(ISNUMBER('工作表1'!U31),'工作表1'!U31,0)</f>
         <v/>
       </c>
+      <c r="S31" s="0">
+        <f>IF('工作表1'!S31="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S31)&gt;0,0,1))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
-      <c r="H32">
+      <c r="H32" s="0">
         <f>IF('工作表1'!D32="","",LEFT('工作表1'!D32,1))</f>
         <v/>
       </c>
-      <c r="I32">
+      <c r="I32" s="0">
         <f>IF(ISNUMBER('工作表1'!F32),'工作表1'!F32,0)</f>
         <v/>
       </c>
-      <c r="J32">
+      <c r="J32" s="0">
+        <f>IF('工作表1'!D32="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D32)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K32" s="0">
         <f>IF('工作表1'!I32="","",LEFT('工作表1'!I32,1))</f>
         <v/>
       </c>
-      <c r="K32">
+      <c r="L32" s="0">
         <f>IF(ISNUMBER('工作表1'!K32),'工作表1'!K32,0)</f>
         <v/>
       </c>
-      <c r="L32">
+      <c r="M32" s="0">
+        <f>IF('工作表1'!I32="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I32)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N32" s="0">
         <f>IF('工作表1'!N32="","",LEFT('工作表1'!N32,1))</f>
         <v/>
       </c>
-      <c r="M32">
+      <c r="O32" s="0">
         <f>IF(ISNUMBER('工作表1'!P32),'工作表1'!P32,0)</f>
         <v/>
       </c>
-      <c r="N32">
+      <c r="P32" s="0">
+        <f>IF('工作表1'!N32="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N32)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q32" s="0">
         <f>IF('工作表1'!S32="","",LEFT('工作表1'!S32,1))</f>
         <v/>
       </c>
-      <c r="O32">
+      <c r="R32" s="0">
         <f>IF(ISNUMBER('工作表1'!U32),'工作表1'!U32,0)</f>
         <v/>
       </c>
+      <c r="S32" s="0">
+        <f>IF('工作表1'!S32="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S32)&gt;0,0,1))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
-      <c r="H33">
+      <c r="H33" s="0">
         <f>IF('工作表1'!D33="","",LEFT('工作表1'!D33,1))</f>
         <v/>
       </c>
-      <c r="I33">
+      <c r="I33" s="0">
         <f>IF(ISNUMBER('工作表1'!F33),'工作表1'!F33,0)</f>
         <v/>
       </c>
-      <c r="J33">
+      <c r="J33" s="0">
+        <f>IF('工作表1'!D33="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D33)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K33" s="0">
         <f>IF('工作表1'!I33="","",LEFT('工作表1'!I33,1))</f>
         <v/>
       </c>
-      <c r="K33">
+      <c r="L33" s="0">
         <f>IF(ISNUMBER('工作表1'!K33),'工作表1'!K33,0)</f>
         <v/>
       </c>
-      <c r="L33">
+      <c r="M33" s="0">
+        <f>IF('工作表1'!I33="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I33)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N33" s="0">
         <f>IF('工作表1'!N33="","",LEFT('工作表1'!N33,1))</f>
         <v/>
       </c>
-      <c r="M33">
+      <c r="O33" s="0">
         <f>IF(ISNUMBER('工作表1'!P33),'工作表1'!P33,0)</f>
         <v/>
       </c>
-      <c r="N33">
+      <c r="P33" s="0">
+        <f>IF('工作表1'!N33="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N33)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q33" s="0">
         <f>IF('工作表1'!S33="","",LEFT('工作表1'!S33,1))</f>
         <v/>
       </c>
-      <c r="O33">
+      <c r="R33" s="0">
         <f>IF(ISNUMBER('工作表1'!U33),'工作表1'!U33,0)</f>
         <v/>
       </c>
+      <c r="S33" s="0">
+        <f>IF('工作表1'!S33="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S33)&gt;0,0,1))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
-      <c r="H34">
-        <f>IF('工作表1'!D34="","",LEFT('工作表1'!D34,1))</f>
-        <v/>
-      </c>
-      <c r="I34">
-        <f>IF(ISNUMBER('工作表1'!F34),'工作表1'!F34,0)</f>
-        <v/>
-      </c>
-      <c r="J34">
-        <f>IF('工作表1'!I34="","",LEFT('工作表1'!I34,1))</f>
-        <v/>
-      </c>
-      <c r="K34">
-        <f>IF(ISNUMBER('工作表1'!K34),'工作表1'!K34,0)</f>
-        <v/>
-      </c>
-      <c r="L34">
-        <f>IF('工作表1'!N34="","",LEFT('工作表1'!N34,1))</f>
-        <v/>
-      </c>
-      <c r="M34">
-        <f>IF(ISNUMBER('工作表1'!P34),'工作表1'!P34,0)</f>
-        <v/>
-      </c>
-      <c r="N34">
-        <f>IF('工作表1'!S34="","",LEFT('工作表1'!S34,1))</f>
-        <v/>
-      </c>
-      <c r="O34">
-        <f>IF(ISNUMBER('工作表1'!U34),'工作表1'!U34,0)</f>
-        <v/>
+      <c r="H34" s="0" t="inlineStr"/>
+      <c r="I34" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="0" t="inlineStr"/>
+      <c r="L34" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="0" t="inlineStr"/>
+      <c r="O34" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="0" t="inlineStr"/>
+      <c r="R34" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
-      <c r="H35">
-        <f>IF('工作表1'!D35="","",LEFT('工作表1'!D35,1))</f>
-        <v/>
-      </c>
-      <c r="I35">
-        <f>IF(ISNUMBER('工作表1'!F35),'工作表1'!F35,0)</f>
-        <v/>
-      </c>
-      <c r="J35">
-        <f>IF('工作表1'!I35="","",LEFT('工作表1'!I35,1))</f>
-        <v/>
-      </c>
-      <c r="K35">
-        <f>IF(ISNUMBER('工作表1'!K35),'工作表1'!K35,0)</f>
-        <v/>
-      </c>
-      <c r="L35">
-        <f>IF('工作表1'!N35="","",LEFT('工作表1'!N35,1))</f>
-        <v/>
-      </c>
-      <c r="M35">
-        <f>IF(ISNUMBER('工作表1'!P35),'工作表1'!P35,0)</f>
-        <v/>
-      </c>
-      <c r="N35">
-        <f>IF('工作表1'!S35="","",LEFT('工作表1'!S35,1))</f>
-        <v/>
-      </c>
-      <c r="O35">
-        <f>IF(ISNUMBER('工作表1'!U35),'工作表1'!U35,0)</f>
-        <v/>
+      <c r="H35" s="0" t="inlineStr"/>
+      <c r="I35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="0" t="inlineStr"/>
+      <c r="L35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="0" t="inlineStr"/>
+      <c r="O35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="0" t="inlineStr"/>
+      <c r="R35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
-      <c r="H36">
-        <f>IF('工作表1'!D36="","",LEFT('工作表1'!D36,1))</f>
-        <v/>
-      </c>
-      <c r="I36">
-        <f>IF(ISNUMBER('工作表1'!F36),'工作表1'!F36,0)</f>
-        <v/>
-      </c>
-      <c r="J36">
-        <f>IF('工作表1'!I36="","",LEFT('工作表1'!I36,1))</f>
-        <v/>
-      </c>
-      <c r="K36">
-        <f>IF(ISNUMBER('工作表1'!K36),'工作表1'!K36,0)</f>
-        <v/>
-      </c>
-      <c r="L36">
-        <f>IF('工作表1'!N36="","",LEFT('工作表1'!N36,1))</f>
-        <v/>
-      </c>
-      <c r="M36">
-        <f>IF(ISNUMBER('工作表1'!P36),'工作表1'!P36,0)</f>
-        <v/>
-      </c>
-      <c r="N36">
-        <f>IF('工作表1'!S36="","",LEFT('工作表1'!S36,1))</f>
-        <v/>
-      </c>
-      <c r="O36">
-        <f>IF(ISNUMBER('工作表1'!U36),'工作表1'!U36,0)</f>
-        <v/>
+      <c r="H36" s="0" t="inlineStr"/>
+      <c r="I36" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="0" t="inlineStr"/>
+      <c r="L36" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="0" t="inlineStr"/>
+      <c r="O36" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="0" t="inlineStr"/>
+      <c r="R36" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
-      <c r="H37">
-        <f>IF('工作表1'!D37="","",LEFT('工作表1'!D37,1))</f>
-        <v/>
-      </c>
-      <c r="I37">
-        <f>IF(ISNUMBER('工作表1'!F37),'工作表1'!F37,0)</f>
-        <v/>
-      </c>
-      <c r="J37">
-        <f>IF('工作表1'!I37="","",LEFT('工作表1'!I37,1))</f>
-        <v/>
-      </c>
-      <c r="K37">
-        <f>IF(ISNUMBER('工作表1'!K37),'工作表1'!K37,0)</f>
-        <v/>
-      </c>
-      <c r="L37">
-        <f>IF('工作表1'!N37="","",LEFT('工作表1'!N37,1))</f>
-        <v/>
-      </c>
-      <c r="M37">
-        <f>IF(ISNUMBER('工作表1'!P37),'工作表1'!P37,0)</f>
-        <v/>
-      </c>
-      <c r="N37">
-        <f>IF('工作表1'!S37="","",LEFT('工作表1'!S37,1))</f>
-        <v/>
-      </c>
-      <c r="O37">
-        <f>IF(ISNUMBER('工作表1'!U37),'工作表1'!U37,0)</f>
-        <v/>
+      <c r="H37" s="0" t="inlineStr"/>
+      <c r="I37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="0" t="inlineStr"/>
+      <c r="L37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="0" t="inlineStr"/>
+      <c r="O37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="0" t="inlineStr"/>
+      <c r="R37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
-      <c r="H38">
-        <f>IF('工作表1'!D38="","",LEFT('工作表1'!D38,1))</f>
-        <v/>
-      </c>
-      <c r="I38">
-        <f>IF(ISNUMBER('工作表1'!F38),'工作表1'!F38,0)</f>
-        <v/>
-      </c>
-      <c r="J38">
-        <f>IF('工作表1'!I38="","",LEFT('工作表1'!I38,1))</f>
-        <v/>
-      </c>
-      <c r="K38">
-        <f>IF(ISNUMBER('工作表1'!K38),'工作表1'!K38,0)</f>
-        <v/>
-      </c>
-      <c r="L38">
-        <f>IF('工作表1'!N38="","",LEFT('工作表1'!N38,1))</f>
-        <v/>
-      </c>
-      <c r="M38">
-        <f>IF(ISNUMBER('工作表1'!P38),'工作表1'!P38,0)</f>
-        <v/>
-      </c>
-      <c r="N38">
-        <f>IF('工作表1'!S38="","",LEFT('工作表1'!S38,1))</f>
-        <v/>
-      </c>
-      <c r="O38">
-        <f>IF(ISNUMBER('工作表1'!U38),'工作表1'!U38,0)</f>
-        <v/>
+      <c r="H38" s="0" t="inlineStr"/>
+      <c r="I38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="0" t="inlineStr"/>
+      <c r="L38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="0" t="inlineStr"/>
+      <c r="O38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="0" t="inlineStr"/>
+      <c r="R38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
-      <c r="H39">
-        <f>IF('工作表1'!D39="","",LEFT('工作表1'!D39,1))</f>
-        <v/>
-      </c>
-      <c r="I39">
-        <f>IF(ISNUMBER('工作表1'!F39),'工作表1'!F39,0)</f>
-        <v/>
-      </c>
-      <c r="J39">
-        <f>IF('工作表1'!I39="","",LEFT('工作表1'!I39,1))</f>
-        <v/>
-      </c>
-      <c r="K39">
-        <f>IF(ISNUMBER('工作表1'!K39),'工作表1'!K39,0)</f>
-        <v/>
-      </c>
-      <c r="L39">
-        <f>IF('工作表1'!N39="","",LEFT('工作表1'!N39,1))</f>
-        <v/>
-      </c>
-      <c r="M39">
-        <f>IF(ISNUMBER('工作表1'!P39),'工作表1'!P39,0)</f>
-        <v/>
-      </c>
-      <c r="N39">
-        <f>IF('工作表1'!S39="","",LEFT('工作表1'!S39,1))</f>
-        <v/>
-      </c>
-      <c r="O39">
-        <f>IF(ISNUMBER('工作表1'!U39),'工作表1'!U39,0)</f>
-        <v/>
+      <c r="H39" s="0" t="inlineStr"/>
+      <c r="I39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="0" t="inlineStr"/>
+      <c r="L39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="0" t="inlineStr"/>
+      <c r="O39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="0" t="inlineStr"/>
+      <c r="R39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
-      <c r="H40">
-        <f>IF('工作表1'!D40="","",LEFT('工作表1'!D40,1))</f>
-        <v/>
-      </c>
-      <c r="I40">
-        <f>IF(ISNUMBER('工作表1'!F40),'工作表1'!F40,0)</f>
-        <v/>
-      </c>
-      <c r="J40">
-        <f>IF('工作表1'!I40="","",LEFT('工作表1'!I40,1))</f>
-        <v/>
-      </c>
-      <c r="K40">
-        <f>IF(ISNUMBER('工作表1'!K40),'工作表1'!K40,0)</f>
-        <v/>
-      </c>
-      <c r="L40">
-        <f>IF('工作表1'!N40="","",LEFT('工作表1'!N40,1))</f>
-        <v/>
-      </c>
-      <c r="M40">
-        <f>IF(ISNUMBER('工作表1'!P40),'工作表1'!P40,0)</f>
-        <v/>
-      </c>
-      <c r="N40">
-        <f>IF('工作表1'!S40="","",LEFT('工作表1'!S40,1))</f>
-        <v/>
-      </c>
-      <c r="O40">
-        <f>IF(ISNUMBER('工作表1'!U40),'工作表1'!U40,0)</f>
-        <v/>
+      <c r="H40" s="0" t="inlineStr"/>
+      <c r="I40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="0" t="inlineStr"/>
+      <c r="L40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="0" t="inlineStr"/>
+      <c r="O40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="0" t="inlineStr"/>
+      <c r="R40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S40" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
-      <c r="H41">
-        <f>IF('工作表1'!D41="","",LEFT('工作表1'!D41,1))</f>
-        <v/>
-      </c>
-      <c r="I41">
-        <f>IF(ISNUMBER('工作表1'!F41),'工作表1'!F41,0)</f>
-        <v/>
-      </c>
-      <c r="J41">
-        <f>IF('工作表1'!I41="","",LEFT('工作表1'!I41,1))</f>
-        <v/>
-      </c>
-      <c r="K41">
-        <f>IF(ISNUMBER('工作表1'!K41),'工作表1'!K41,0)</f>
-        <v/>
-      </c>
-      <c r="L41">
-        <f>IF('工作表1'!N41="","",LEFT('工作表1'!N41,1))</f>
-        <v/>
-      </c>
-      <c r="M41">
-        <f>IF(ISNUMBER('工作表1'!P41),'工作表1'!P41,0)</f>
-        <v/>
-      </c>
-      <c r="N41">
-        <f>IF('工作表1'!S41="","",LEFT('工作表1'!S41,1))</f>
-        <v/>
-      </c>
-      <c r="O41">
-        <f>IF(ISNUMBER('工作表1'!U41),'工作表1'!U41,0)</f>
-        <v/>
+      <c r="H41" s="0" t="inlineStr"/>
+      <c r="I41" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="0" t="inlineStr"/>
+      <c r="L41" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="0" t="inlineStr"/>
+      <c r="O41" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="0" t="inlineStr"/>
+      <c r="R41" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S41" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
-      <c r="H42">
+      <c r="H42" s="0">
         <f>IF('工作表1'!D42="","",LEFT('工作表1'!D42,1))</f>
         <v/>
       </c>
-      <c r="I42">
+      <c r="I42" s="0">
         <f>IF(ISNUMBER('工作表1'!F42),'工作表1'!F42,0)</f>
         <v/>
       </c>
-      <c r="J42">
+      <c r="J42" s="0">
+        <f>IF('工作表1'!D42="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D42)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K42" s="0">
         <f>IF('工作表1'!I42="","",LEFT('工作表1'!I42,1))</f>
         <v/>
       </c>
-      <c r="K42">
+      <c r="L42" s="0">
         <f>IF(ISNUMBER('工作表1'!K42),'工作表1'!K42,0)</f>
         <v/>
       </c>
-      <c r="L42">
+      <c r="M42" s="0">
+        <f>IF('工作表1'!I42="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I42)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N42" s="0">
         <f>IF('工作表1'!N42="","",LEFT('工作表1'!N42,1))</f>
         <v/>
       </c>
-      <c r="M42">
+      <c r="O42" s="0">
         <f>IF(ISNUMBER('工作表1'!P42),'工作表1'!P42,0)</f>
         <v/>
       </c>
-      <c r="N42">
+      <c r="P42" s="0">
+        <f>IF('工作表1'!N42="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N42)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q42" s="0">
         <f>IF('工作表1'!S42="","",LEFT('工作表1'!S42,1))</f>
         <v/>
       </c>
-      <c r="O42">
+      <c r="R42" s="0">
         <f>IF(ISNUMBER('工作表1'!U42),'工作表1'!U42,0)</f>
         <v/>
       </c>
+      <c r="S42" s="0">
+        <f>IF('工作表1'!S42="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S42)&gt;0,0,1))</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
-      <c r="H43">
+      <c r="H43" s="0">
         <f>IF('工作表1'!D43="","",LEFT('工作表1'!D43,1))</f>
         <v/>
       </c>
-      <c r="I43">
+      <c r="I43" s="0">
         <f>IF(ISNUMBER('工作表1'!F43),'工作表1'!F43,0)</f>
         <v/>
       </c>
-      <c r="J43">
+      <c r="J43" s="0">
+        <f>IF('工作表1'!D43="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D43)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K43" s="0">
         <f>IF('工作表1'!I43="","",LEFT('工作表1'!I43,1))</f>
         <v/>
       </c>
-      <c r="K43">
+      <c r="L43" s="0">
         <f>IF(ISNUMBER('工作表1'!K43),'工作表1'!K43,0)</f>
         <v/>
       </c>
-      <c r="L43">
+      <c r="M43" s="0">
+        <f>IF('工作表1'!I43="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I43)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N43" s="0">
         <f>IF('工作表1'!N43="","",LEFT('工作表1'!N43,1))</f>
         <v/>
       </c>
-      <c r="M43">
+      <c r="O43" s="0">
         <f>IF(ISNUMBER('工作表1'!P43),'工作表1'!P43,0)</f>
         <v/>
       </c>
-      <c r="N43">
+      <c r="P43" s="0">
+        <f>IF('工作表1'!N43="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N43)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q43" s="0">
         <f>IF('工作表1'!S43="","",LEFT('工作表1'!S43,1))</f>
         <v/>
       </c>
-      <c r="O43">
+      <c r="R43" s="0">
         <f>IF(ISNUMBER('工作表1'!U43),'工作表1'!U43,0)</f>
         <v/>
       </c>
+      <c r="S43" s="0">
+        <f>IF('工作表1'!S43="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S43)&gt;0,0,1))</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
-      <c r="H44">
+      <c r="H44" s="0">
         <f>IF('工作表1'!D44="","",LEFT('工作表1'!D44,1))</f>
         <v/>
       </c>
-      <c r="I44">
+      <c r="I44" s="0">
         <f>IF(ISNUMBER('工作表1'!F44),'工作表1'!F44,0)</f>
         <v/>
       </c>
-      <c r="J44">
+      <c r="J44" s="0">
+        <f>IF('工作表1'!D44="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D44)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K44" s="0">
         <f>IF('工作表1'!I44="","",LEFT('工作表1'!I44,1))</f>
         <v/>
       </c>
-      <c r="K44">
+      <c r="L44" s="0">
         <f>IF(ISNUMBER('工作表1'!K44),'工作表1'!K44,0)</f>
         <v/>
       </c>
-      <c r="L44">
+      <c r="M44" s="0">
+        <f>IF('工作表1'!I44="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I44)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N44" s="0">
         <f>IF('工作表1'!N44="","",LEFT('工作表1'!N44,1))</f>
         <v/>
       </c>
-      <c r="M44">
+      <c r="O44" s="0">
         <f>IF(ISNUMBER('工作表1'!P44),'工作表1'!P44,0)</f>
         <v/>
       </c>
-      <c r="N44">
+      <c r="P44" s="0">
+        <f>IF('工作表1'!N44="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N44)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q44" s="0">
         <f>IF('工作表1'!S44="","",LEFT('工作表1'!S44,1))</f>
         <v/>
       </c>
-      <c r="O44">
+      <c r="R44" s="0">
         <f>IF(ISNUMBER('工作表1'!U44),'工作表1'!U44,0)</f>
         <v/>
       </c>
+      <c r="S44" s="0">
+        <f>IF('工作表1'!S44="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S44)&gt;0,0,1))</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
-      <c r="H45">
+      <c r="H45" s="0">
         <f>IF('工作表1'!D45="","",LEFT('工作表1'!D45,1))</f>
         <v/>
       </c>
-      <c r="I45">
+      <c r="I45" s="0">
         <f>IF(ISNUMBER('工作表1'!F45),'工作表1'!F45,0)</f>
         <v/>
       </c>
-      <c r="J45">
+      <c r="J45" s="0">
+        <f>IF('工作表1'!D45="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D45)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K45" s="0">
         <f>IF('工作表1'!I45="","",LEFT('工作表1'!I45,1))</f>
         <v/>
       </c>
-      <c r="K45">
+      <c r="L45" s="0">
         <f>IF(ISNUMBER('工作表1'!K45),'工作表1'!K45,0)</f>
         <v/>
       </c>
-      <c r="L45">
+      <c r="M45" s="0">
+        <f>IF('工作表1'!I45="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I45)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N45" s="0">
         <f>IF('工作表1'!N45="","",LEFT('工作表1'!N45,1))</f>
         <v/>
       </c>
-      <c r="M45">
+      <c r="O45" s="0">
         <f>IF(ISNUMBER('工作表1'!P45),'工作表1'!P45,0)</f>
         <v/>
       </c>
-      <c r="N45">
+      <c r="P45" s="0">
+        <f>IF('工作表1'!N45="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N45)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q45" s="0">
         <f>IF('工作表1'!S45="","",LEFT('工作表1'!S45,1))</f>
         <v/>
       </c>
-      <c r="O45">
+      <c r="R45" s="0">
         <f>IF(ISNUMBER('工作表1'!U45),'工作表1'!U45,0)</f>
         <v/>
       </c>
+      <c r="S45" s="0">
+        <f>IF('工作表1'!S45="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S45)&gt;0,0,1))</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
-      <c r="H46">
+      <c r="H46" s="0">
         <f>IF('工作表1'!D46="","",LEFT('工作表1'!D46,1))</f>
         <v/>
       </c>
-      <c r="I46">
+      <c r="I46" s="0">
         <f>IF(ISNUMBER('工作表1'!F46),'工作表1'!F46,0)</f>
         <v/>
       </c>
-      <c r="J46">
+      <c r="J46" s="0">
+        <f>IF('工作表1'!D46="",0,IF(COUNTIF('工作表1'!$C$50:$C$68,'工作表1'!D46)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="K46" s="0">
         <f>IF('工作表1'!I46="","",LEFT('工作表1'!I46,1))</f>
         <v/>
       </c>
-      <c r="K46">
+      <c r="L46" s="0">
         <f>IF(ISNUMBER('工作表1'!K46),'工作表1'!K46,0)</f>
         <v/>
       </c>
-      <c r="L46">
+      <c r="M46" s="0">
+        <f>IF('工作表1'!I46="",0,IF(COUNTIF('工作表1'!$H$50:$H$68,'工作表1'!I46)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="N46" s="0">
         <f>IF('工作表1'!N46="","",LEFT('工作表1'!N46,1))</f>
         <v/>
       </c>
-      <c r="M46">
+      <c r="O46" s="0">
         <f>IF(ISNUMBER('工作表1'!P46),'工作表1'!P46,0)</f>
         <v/>
       </c>
-      <c r="N46">
+      <c r="P46" s="0">
+        <f>IF('工作表1'!N46="",0,IF(COUNTIF('工作表1'!$M$50:$M$68,'工作表1'!N46)&gt;0,0,1))</f>
+        <v/>
+      </c>
+      <c r="Q46" s="0">
         <f>IF('工作表1'!S46="","",LEFT('工作表1'!S46,1))</f>
         <v/>
       </c>
-      <c r="O46">
+      <c r="R46" s="0">
         <f>IF(ISNUMBER('工作表1'!U46),'工作表1'!U46,0)</f>
         <v/>
       </c>
+      <c r="S46" s="0">
+        <f>IF('工作表1'!S46="",0,IF(COUNTIF('工作表1'!$R$50:$R$68,'工作表1'!S46)&gt;0,0,1))</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
-      <c r="H47">
-        <f>IF('工作表1'!D47="","",LEFT('工作表1'!D47,1))</f>
-        <v/>
-      </c>
-      <c r="I47">
-        <f>IF(ISNUMBER('工作表1'!F47),'工作表1'!F47,0)</f>
-        <v/>
-      </c>
-      <c r="J47">
-        <f>IF('工作表1'!I47="","",LEFT('工作表1'!I47,1))</f>
-        <v/>
-      </c>
-      <c r="K47">
-        <f>IF(ISNUMBER('工作表1'!K47),'工作表1'!K47,0)</f>
-        <v/>
-      </c>
-      <c r="L47">
-        <f>IF('工作表1'!N47="","",LEFT('工作表1'!N47,1))</f>
-        <v/>
-      </c>
-      <c r="M47">
-        <f>IF(ISNUMBER('工作表1'!P47),'工作表1'!P47,0)</f>
-        <v/>
-      </c>
-      <c r="N47">
-        <f>IF('工作表1'!S47="","",LEFT('工作表1'!S47,1))</f>
-        <v/>
-      </c>
-      <c r="O47">
-        <f>IF(ISNUMBER('工作表1'!U47),'工作表1'!U47,0)</f>
-        <v/>
+      <c r="H47" s="0" t="inlineStr"/>
+      <c r="I47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="0" t="inlineStr"/>
+      <c r="L47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="0" t="inlineStr"/>
+      <c r="O47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="0" t="inlineStr"/>
+      <c r="R47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S47" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove review comments and highlight fills from corrected workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011perRKT2EmENmrFmt59Nd9
</commit_message>
<xml_diff>
--- a/BIM分錄_檢核修正版.xlsx
+++ b/BIM分錄_檢核修正版.xlsx
@@ -1554,391 +1554,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>檢核</author>
-  </authors>
-  <commentList>
-    <comment ref="F21" authorId="0" shapeId="0">
-      <text>
-        <t>修正：原寫死5；毛利=收入105.26-成本100=5.26，寫死使本筆借貸差0.263</t>
-      </text>
-    </comment>
-    <comment ref="K21" authorId="0" shapeId="0">
-      <text>
-        <t>修正：同F21</t>
-      </text>
-    </comment>
-    <comment ref="E50" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C50,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J50" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H50,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O50" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M50,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T50" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R50,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E51" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C51,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J51" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H51,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O51" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M51,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T51" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R51,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E52" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$34,$C52,$F$2:$F$34)</t>
-      </text>
-    </comment>
-    <comment ref="J52" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$34,$H52,$K$2:$K$34)</t>
-      </text>
-    </comment>
-    <comment ref="O52" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$34,$M52,$P$2:$P$34)</t>
-      </text>
-    </comment>
-    <comment ref="T52" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$34,$R52,$U$2:$U$34)</t>
-      </text>
-    </comment>
-    <comment ref="E53" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C53,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J53" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H53,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O53" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M53,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T53" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R53,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E54" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C54,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J54" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H54,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O54" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M54,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T54" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R54,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E55" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C55,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J55" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H55,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O55" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M55,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T55" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R55,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E56" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C56,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J56" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H56,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O56" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M56,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T56" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R56,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E57" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C57,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J57" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H57,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O57" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M57,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T57" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R57,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E58" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C58,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J58" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H58,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O58" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M58,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T58" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R58,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E59" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C59,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J59" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H59,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O59" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$34,$M59,$P$2:$P$34)</t>
-      </text>
-    </comment>
-    <comment ref="T59" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$34,$R59,$U$2:$U$34)</t>
-      </text>
-    </comment>
-    <comment ref="E60" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C60,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J60" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H60,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O60" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M60,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T60" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R60,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="J61" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H61,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O61" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M61,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T61" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R61,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E62" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C62,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J62" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H62,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O62" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$36,$M62,$P$2:$P$36)</t>
-      </text>
-    </comment>
-    <comment ref="T62" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$36,$R62,$U$2:$U$36)</t>
-      </text>
-    </comment>
-    <comment ref="E63" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C63,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J63" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H63,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O63" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M63,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T63" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R63,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="J64" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H64,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O64" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M64,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T64" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R64,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="J65" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H65,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O65" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M65,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T65" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$37,$R65,$U$2:$U$37)</t>
-      </text>
-    </comment>
-    <comment ref="E66" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C66,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J66" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H66,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O66" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M66,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T66" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R66,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E67" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C67,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J67" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H67,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O67" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M67,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T67" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R67,$U$2:$U$47)</t>
-      </text>
-    </comment>
-    <comment ref="E68" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($D$2:$D$47,$C68,$F$2:$F$47)</t>
-      </text>
-    </comment>
-    <comment ref="J68" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($I$2:$I$47,$H68,$K$2:$K$47)</t>
-      </text>
-    </comment>
-    <comment ref="O68" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($N$2:$N$47,$M68,$P$2:$P$47)</t>
-      </text>
-    </comment>
-    <comment ref="T68" authorId="0" shapeId="0">
-      <text>
-        <t>修正：只加BIM分錄列(4-10,16-22,31-33,42-46)，排除ELIA/TBU列。原式 =SUMIF($S$2:$S$47,$R68,$U$2:$U$47)</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3388,7 +3003,7 @@
           <t>在建損益-承攬案</t>
         </is>
       </c>
-      <c r="F21" s="177">
+      <c r="F21" s="1">
         <f>-F22-F20</f>
         <v/>
       </c>
@@ -3406,7 +3021,7 @@
           <t>在建損益-承攬案</t>
         </is>
       </c>
-      <c r="K21" s="177">
+      <c r="K21" s="1">
         <f>-K22-K20</f>
         <v/>
       </c>
@@ -4721,7 +4336,7 @@
           <t>在建損益-承攬案</t>
         </is>
       </c>
-      <c r="E51" s="198">
+      <c r="E51" s="79">
         <f>SUMIF($D$4:$D$10,$C51,$F$4:$F$10)+SUMIF($D$16:$D$22,$C51,$F$16:$F$22)+SUMIF($D$31:$D$33,$C51,$F$31:$F$33)+SUMIF($D$42:$D$46,$C51,$F$42:$F$46)</f>
         <v/>
       </c>
@@ -5293,7 +4908,7 @@
           <t>承攬工程收入</t>
         </is>
       </c>
-      <c r="E58" s="198">
+      <c r="E58" s="86">
         <f>SUMIF($D$4:$D$10,$C58,$F$4:$F$10)+SUMIF($D$16:$D$22,$C58,$F$16:$F$22)+SUMIF($D$31:$D$33,$C58,$F$31:$F$33)+SUMIF($D$42:$D$46,$C58,$F$42:$F$46)</f>
         <v/>
       </c>
@@ -5381,7 +4996,7 @@
           <t>承攬工程成本</t>
         </is>
       </c>
-      <c r="E59" s="198">
+      <c r="E59" s="86">
         <f>SUMIF($D$4:$D$10,$C59,$F$4:$F$10)+SUMIF($D$16:$D$22,$C59,$F$16:$F$22)+SUMIF($D$31:$D$33,$C59,$F$31:$F$33)+SUMIF($D$42:$D$46,$C59,$F$42:$F$46)</f>
         <v/>
       </c>
@@ -5475,7 +5090,7 @@
           <t>專案成本</t>
         </is>
       </c>
-      <c r="T60" s="198">
+      <c r="T60" s="86">
         <f>SUMIF($S$4:$S$10,$R60,$U$4:$U$10)+SUMIF($S$16:$S$22,$R60,$U$16:$U$22)+SUMIF($S$31:$S$33,$R60,$U$31:$U$33)+SUMIF($S$42:$S$46,$R60,$U$42:$U$46)</f>
         <v/>
       </c>
@@ -5685,7 +5300,7 @@
           <t>人事分攤</t>
         </is>
       </c>
-      <c r="T64" s="198">
+      <c r="T64" s="86">
         <f>SUMIF($S$4:$S$10,$R64,$U$4:$U$10)+SUMIF($S$16:$S$22,$R64,$U$16:$U$22)+SUMIF($S$31:$S$33,$R64,$U$31:$U$33)+SUMIF($S$42:$S$46,$R64,$U$42:$U$46)</f>
         <v/>
       </c>
@@ -5778,7 +5393,7 @@
           <t>電腦out charge</t>
         </is>
       </c>
-      <c r="T66" s="198">
+      <c r="T66" s="86">
         <f>SUMIF($S$4:$S$10,$R66,$U$4:$U$10)+SUMIF($S$16:$S$22,$R66,$U$16:$U$22)+SUMIF($S$31:$S$33,$R66,$U$31:$U$33)+SUMIF($S$42:$S$46,$R66,$U$42:$U$46)</f>
         <v/>
       </c>
@@ -5956,6 +5571,8 @@
         <v/>
       </c>
     </row>
+    <row r="70"/>
+    <row r="71"/>
     <row r="72" ht="16.2" customHeight="1" s="168" thickBot="1"/>
     <row r="73" ht="16.2" customHeight="1" s="168" thickTop="1">
       <c r="C73" s="2" t="inlineStr">
@@ -6086,7 +5703,6 @@
     <mergeCell ref="F50:F52"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>